<commit_message>
Rebuild the naming workbook as a standalone shareable document
The previous version held the findings but not the evidence, so anyone opening
it cold had to take the conclusions on trust. It now carries its own sources.

Four sheets: "Start here" leads with the recommendation and ranks all twelve
searched names best to worst with their sample mark; "Findings and sources"
gives the full finding per name alongside the URLs to check it; "All 100
candidates" keeps the numbering used on the shared naming page; "Screened out"
records the patterns avoided and the clearance caveat.

All twelve now appear, including the three ruled out, because the story is that
twelve were checked rather than that nine survived. Trailhead and Rally Point
carry no mark, labelled as ruled out, since drawing logos for names that are
legally blocked would be misleading.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/share/VetPath-Naming-Candidates.xlsx
+++ b/share/VetPath-Naming-Candidates.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top 10 + logos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All 100 names" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screened out" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start here" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings and sources" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All 100 candidates" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screened out" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="20">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,6 +40,11 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="000F6E56"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
@@ -47,9 +53,15 @@
       <sz val="9"/>
     </font>
     <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <color rgb="0016324D"/>
+      <sz val="12"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="000F6E56"/>
-      <sz val="10"/>
+      <sz val="9.5"/>
     </font>
     <font>
       <color rgb="001B2A3A"/>
@@ -58,25 +70,30 @@
     <font>
       <b val="1"/>
       <color rgb="0040506A"/>
-      <sz val="10"/>
+      <sz val="9.5"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="008A5A10"/>
-      <sz val="10"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="005A6B7B"/>
+      <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="009C2A16"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="10.5"/>
+      <sz val="9.5"/>
     </font>
     <font>
       <color rgb="001B2A3A"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="00185FA5"/>
+      <sz val="8.5"/>
     </font>
     <font>
       <b val="1"/>
@@ -89,11 +106,11 @@
       <sz val="10.5"/>
     </font>
     <font>
+      <b val="1"/>
+      <color rgb="009C2A16"/>
       <sz val="10.5"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="009C2A16"/>
       <sz val="10.5"/>
     </font>
     <font>
@@ -103,12 +120,12 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="005A6B7B"/>
-      <sz val="10.5"/>
+      <color rgb="0016324D"/>
+      <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="0016324D"/>
+      <color rgb="009C2A16"/>
       <sz val="10"/>
     </font>
     <font>
@@ -116,7 +133,7 @@
       <sz val="9.5"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -148,11 +165,6 @@
         <fgColor rgb="00FBE9E7"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2F4F7"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -180,55 +192,81 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -313,7 +351,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>4</row>
+      <row>5</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="2238375" cy="647700"/>
@@ -338,7 +376,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>5</row>
+      <row>6</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="2238375" cy="647700"/>
@@ -363,7 +401,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>6</row>
+      <row>7</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="2238375" cy="647700"/>
@@ -388,7 +426,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>7</row>
+      <row>8</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="2238375" cy="647700"/>
@@ -413,7 +451,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>8</row>
+      <row>9</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="2238375" cy="647700"/>
@@ -438,7 +476,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>9</row>
+      <row>10</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="2238375" cy="647700"/>
@@ -463,7 +501,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>10</row>
+      <row>11</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="2238375" cy="647700"/>
@@ -488,7 +526,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>11</row>
+      <row>12</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="2238375" cy="647700"/>
@@ -513,7 +551,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>12</row>
+      <row>13</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="2238375" cy="647700"/>
@@ -538,7 +576,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>13</row>
+      <row>16</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="2238375" cy="647700"/>
@@ -851,224 +889,330 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="72" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="64" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Naming the platform: top 10 with sample marks</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1">
+          <t>Naming the platform: where it stands</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="52" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sample logos only, drawn to show how each name behaves as a mark. Not final identity work. All ten have now been searched. Statuses come from a preliminary public-record search on 29 July 2026, not a legal clearance. Trailhead and Rally Point are absent because live federal registrations block them.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+          <t>Twelve candidates searched against public domain and USPTO records on 29 July 2026, ranked best to worst. Sample marks show how a name behaves as a logo; they are not final identity work. IMPORTANT: this is a preliminary search of public records, NOT a legal clearance opinion. USPTO full-text search blocked automated access, so registrations were pulled one at a time and coverage is partial. Absence of a conflict means nothing was found, not that nothing exists. No WHOIS was run, so nothing here says a domain is available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="42" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>RECOMMENDATION: take Due North and Lodestar to the table. They are the two cleanest, and for the same reason: they carry the least military flavour. The pattern across all twelve is that the more evocative the military reference, the more crowded the name turned out to be.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Sample mark</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Name / status</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Where it stands</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="62" customHeight="1">
-      <c r="A5" s="4" t="n">
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>The headline</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="62" customHeight="1">
+      <c r="A6" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>Due North
-CLEANEST OVERALL</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>Zero veteran-space collisions. The .com is gone and it will be misheard as True North.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="62" customHeight="1">
-      <c r="A6" s="4" t="n">
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Due North</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>CLEANEST OVERALL</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Zero veteran-space collisions, the only such result of the twelve.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="62" customHeight="1">
+      <c r="A7" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>Lodestar
-CLEANEST VET SPACE</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>No veteran org, transition program or military tool found using it. Live Cl. 9 and Cl. 36 marks; .com is an insurance TPA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="62" customHeight="1">
-      <c r="A7" s="4" t="n">
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Lodestar</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>CLEANEST VETERAN SPACE</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>No veteran nonprofit, transition program or military tool found using it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="62" customHeight="1">
+      <c r="A8" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>After Action
-USABLE, WITH DRAG</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>No blocking registration found. Weakly distinctive; crowded with veteran media.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="62" customHeight="1">
-      <c r="A8" s="4" t="n">
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>After Action</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>USABLE, WITH DRAG</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Cleanest trademark result: no live registered mark found blocking our classes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="62" customHeight="1">
+      <c r="A9" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="5" t="inlineStr"/>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>Earned
-USABLE, WITH DRAG</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>Clean on paper. earned.com is a $3.9B wealth firm; 'earned benefits' kills organic search.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="62" customHeight="1">
-      <c r="A9" s="4" t="n">
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Earned</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>USABLE, WITH DRAG</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>No blocking registration and no veteran-space entity, but the .com and search are problems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="62" customHeight="1">
+      <c r="A10" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="5" t="inlineStr"/>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>First Light
-USABLE, WITH DRAG</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>Nobody owns it in our lane, but we would be the twentieth FirstLight. Four live Cl. 36 marks.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="62" customHeight="1">
-      <c r="A10" s="4" t="n">
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>First Light</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>USABLE, WITH DRAG</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Crowded but diffusely: nobody owns it in veteran benefits or career planning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="62" customHeight="1">
+      <c r="A11" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="5" t="inlineStr"/>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>Muster
-HIGH RISK</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>Echelon Front holds an incontestable Class 41. Orion Talent launched Muster(TM) for veteran hiring.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="62" customHeight="1">
-      <c r="A11" s="4" t="n">
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Muster</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>HIGH RISK</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Blocked by an incontestable Class 41 registration, and a veteran-hiring platform launched under it in 2025.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="62" customHeight="1">
+      <c r="A12" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="5" t="inlineStr"/>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>Waypoint
-HIGH RISK</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>Sandboxx already ships 'Waypoints' to the same users. The .com is a debt collector.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="62" customHeight="1">
-      <c r="A12" s="4" t="n">
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Waypoint</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>HIGH RISK</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>A near-identical military life app already ships to the same users.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="62" customHeight="1">
+      <c r="A13" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="5" t="inlineStr"/>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>Reveille
-HIGH RISK</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>Three veteran orgs, one with a live Class 41 registration. Texas A&amp;M overhang.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="62" customHeight="1">
-      <c r="A13" s="4" t="n">
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Reveille</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>HIGH RISK</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>Three veteran organisations use it, one holding a live registration in our class.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="62" customHeight="1">
+      <c r="A14" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="5" t="inlineStr"/>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>Azimuth
-HIGH RISK</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>Register is clear, but 'Azimuth Check' is a US Army assessment and four veteran orgs use it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="62" customHeight="1">
-      <c r="A14" s="4" t="n">
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Azimuth</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>HIGH RISK</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>The register is clear, which is the trap. The US Army already uses the phrase.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="62" customHeight="1">
+      <c r="A15" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="5" t="inlineStr"/>
-      <c r="C14" s="10" t="inlineStr">
-        <is>
-          <t>Squared Away
-RULE OUT</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>squaredawayvet.org is already our product under this name. Every class occupied.</t>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>no mark drawn
+(ruled out)</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Trailhead</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>RULE OUT</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>Salesforce owns the word in exactly our two classes, and runs a veteran programme under it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="62" customHeight="1">
+      <c r="A16" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>no mark drawn
+(ruled out)</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Rally Point</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>RULE OUT</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>Five live incontestable registrations describing our product in trademark language.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="62" customHeight="1">
+      <c r="A17" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Squared Away</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>RULE OUT</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>Someone is already running this exact product under this exact name.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:D2"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1076,6 +1220,363 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="96" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>What the search found, and where to check it</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="44" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Every claim below can be checked at the sources in the last column. Where a registration number is given it was read on the USPTO record. Domains were loaded directly to see what they serve.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>What was found</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Sources (open in a browser)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="118" customHeight="1">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>Due North</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>CLEANEST OVERALL</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Searches pairing Due North with veterans, military and transition returned no organisation operating in this space. It is not clean, only cleanest. duenorth.com 301-redirects to aeritekna.com, a private-equity-backed refrigeration manufacturer that acquired Due North in 2025, so the domain is unobtainable. SureWerx sells Due North(R) ice cleats using the registered symbol. A live Class 45 registration (Reg. 6634132) covers legal services. It will also be misheard as True North, which is an active US veterans nonprofit.</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="inlineStr">
+        <is>
+          <t>duenorth.com
+duenorthproducts.com
+duenorthtulsa.org
+aeritekna.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="118" customHeight="1">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>Lodestar</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>CLEANEST VETERAN SPACE</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>Three targeted searches found nothing in the veteran space except an internal employee resource group at a consulting firm, which our users would never encounter. The problems are the ordinary kind: a live Class 9 registration on the bare word (Reg. 7006981, owned by a game studio, so a different field of use), a live Class 36 for investment advisory, and pending Class 41 and 42 filings. lodestar.com is a national insurance claims administrator under Old Republic that rebranded onto it in 2026. Note for Kaleb: Lodestar is heavily used across insurance.</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="inlineStr">
+        <is>
+          <t>lodestar.com
+insurancejournal.com/news/midwest/2026/04/13/865643.htm
+trademarkelite.com/trademark/trademark-detail/90477866/LODESTAR
+lodestarcs.com/military</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="118" customHeight="1">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>After Action</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>USABLE, WITH DRAG</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Nothing live and registered was found in Classes 9, 35, 36, 41, 42 or 45. The one veteran-space Class 41 filing was abandoned in 2016. The drag is practical rather than legal: 'after action review' is military doctrine, so the name is weakly distinctive and hard to defend or own in search. At least four veteran media brands already use it, including a PBS-distributed documentary series. afteraction.com does not resolve. The former After Action Network let its .org lapse to an adult-content site, which is a live brand-safety hazard attached to the phrase.</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="inlineStr">
+        <is>
+          <t>afteractionshow.org
+trademarks.justia.com/866/92/after-action-86692165.html
+news.va.gov/75974/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="118" customHeight="1">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Earned</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>USABLE, WITH DRAG</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>No plain-word EARNED registration surfaced in our classes and no veteran organisation uses it. However earned.com belongs to Earned Wealth, which has raised $200M, manages $3.9B, runs a consumer finance app and filed three new marks in 2026: a veteran financial-planning tool sits closer to their lane than is comfortable, and they can afford to send letters. Separately, 'earned benefits' is standard VA vocabulary across nearly every veteran page on the internet, which makes organic discovery extremely hard.</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="inlineStr">
+        <is>
+          <t>earned.com
+uspto.report/company/Earned-Wealth-Operating-Company-Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="118" customHeight="1">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>First Light</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>USABLE, WITH DRAG</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>We would be roughly the twentieth FirstLight in America. firstlight.com is a stock photography company and firstlight.net is a regional fiber telecom. Class 36 has four separate live registrations, one of them FirstLight Federal Credit Union, which serves Fort Bliss and runs a Veterans Benefits Banking Program. Class 42 has two live SaaS registrations and Class 9 has an active one (Aurora). No single fatal blocker, but a permanent disambiguation tax.</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>firstlight.com
+firstlight.net
+firstlightfcu.org
+firstlight-usa.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="118" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Muster</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>HIGH RISK</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>Echelon Front (Jocko Willink's company) holds MUSTER, Reg. 5611610, live and incontestable as of February 2025, in Class 41 for business education and training. Orion Talent launched Muster(TM) on Veterans Day 2025 connecting employers to transitioning service members. Adyton ships 'Mustr' to four service branches. A new Class 9 application for military-themed social software was filed in May 2026 and is pending. www.muster.com is an advocacy SaaS company. Being ordinary military vocabulary cuts twice: the space is crowded and we could never own it strongly.</t>
+        </is>
+      </c>
+      <c r="D10" s="17" t="inlineStr">
+        <is>
+          <t>tsdr.uspto.gov/statusview/sn87871302
+oriontalent.com/solutions/muster/
+getmustr.app
+muster.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="118" customHeight="1">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>Waypoint</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>HIGH RISK</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Sandboxx ships 'Waypoints', covering rank progression, MOS insights, a TSP calculator and a PCS calculator, on iOS, Android and web: same product shape, same user, one letter apart. A live Class 9 registration (Reg. 5891296) covers downloadable guides and legal and business forms, which is close to a benefits-and-forms planner. DSPII Waypoint does VA benefits, employment and housing for veterans, which is our three pillars exactly. And waypoint.com is a debt collection agency, so veterans searching the name land on a collections firm.</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="inlineStr">
+        <is>
+          <t>sandboxx.us/waypoints/
+tsdr.uspto.gov/statusview/sn88398836
+dspwaypoint.org
+waypointvets.org
+waypoint.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="118" customHeight="1">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Reveille</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>HIGH RISK</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>Reveille and Retreat Project holds Reg. 8164652, live, Class 41, for education covering female veterans, female service members and their families. The Reveille Foundation runs veteran housing and employment programmes with Department of Labor and VA ties. Reveille Grounds is a veteran coworking hub in Baltimore. Reveille Executive Coaching holds a live Class 41 career-coaching registration. Texas A&amp;M's mascot claim is a separate overhang, and reveille.com has belonged to a web services firm since 1991.</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>reveilleandretreatproject.org
+reveillefoundation.org
+reveille.com
+tamu.edu/statements/trademark.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="118" customHeight="1">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>Azimuth</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>HIGH RISK</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Every Azimuth registration in Classes 9, 36, 41 and 42 is cancelled or abandoned, because the term is too generic in this domain for anyone to hold. Meanwhile 'Azimuth Check' is the name of a US Army soldier well-being assessment; GallantFew runs an Azimuth Check assessment; the Azimuth Check Foundation serves injured veterans; and Transition Azimuth Check (TrAC) is a military-to-civilian transition programme for special operations members. For a product positioned as 'not the VA, not the government', sharing a name with an Army assessment tool actively undercuts it. azimuth.org was a veteran resource-connector nonprofit doing our exact job and now bounces to a parking lander, making it a dormant prior-use claim rather than a clear field.</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>armyresilience.army.mil
+gallantfew.org/azimuthcheck
+thestationfoundation.org/trac/
+azimuthcheckfoundation.org
+azimuth.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="118" customHeight="1">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>Trailhead</t>
+        </is>
+      </c>
+      <c r="B14" s="20" t="inlineStr">
+        <is>
+          <t>RULE OUT</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>TRAILHEAD, Reg. 5115199, live, standard character, owner salesforce.com inc., Classes 41 and 42, covering 'e-learning platforms' and 'learning management systems'. Confirmed directly on the USPTO record. trailhead.com redirects to trailhead.salesforce.com. Salesforce also runs Trailhead Military, free training and certification for veterans and military spouses, under that mark. And Project Trailhead already exists: a veteran-founded transition app whose tagline is 'Your Civilian Mission Starts Here'.</t>
+        </is>
+      </c>
+      <c r="D14" s="17" t="inlineStr">
+        <is>
+          <t>trailhead.salesforce.com
+trademarks.justia.com/865/88/trailhead-86588816.html
+projecttrailhead.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="118" customHeight="1">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>Rally Point</t>
+        </is>
+      </c>
+      <c r="B15" s="20" t="inlineStr">
+        <is>
+          <t>RULE OUT</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>RallyPoint Networks holds five live registrations across Classes 35, 38, 41 and 45. Reg. 4730603 covers 'a website containing employment information and listings on career and job opportunities for military personnel' and 'training information on career and job opportunities for military personnel'. Section 15 declarations were accepted, so the marks are incontestable and cannot be attacked as merely descriptive. Counsel is Latham &amp; Watkins and they have already beaten a cancellation attempt. At least five other veteran organisations use the name. Their site has been down since around March 2026, which does not free the name: the registrations run for years.</t>
+        </is>
+      </c>
+      <c r="D15" s="17" t="inlineStr">
+        <is>
+          <t>trademarks.justia.com/855/81/rallypoint-85581784.html
+trademarks.justia.com/863/42/rp-rallypoint-86342578.html
+en.wikipedia.org/wiki/RallyPoint
+operationrallypoint.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="118" customHeight="1">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>Squared Away</t>
+        </is>
+      </c>
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>RULE OUT</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>squaredawayvet.org is live today and describes itself as 'your personal Hub for Veteran resources and documents', with pages for Documents, Education Benefits, Service Connection, Communities and Colleges. Confirmed by loading it. First Command, a 68-year-old military financial firm, holds a live Class 36 registration on SQUARED AWAY and markets 'Get Your Finances Squared Away' to service members. The military-spouse staffing company Squared Away made the Inc. 5000. Two further applications are in prosecution: Class 9 for software organising military personnel, and a multi-class filing for a veteran app. Every class we occupy has a live or pending mark, and because the phrase is ordinary military slang, distinctiveness is unreachable.</t>
+        </is>
+      </c>
+      <c r="D16" s="17" t="inlineStr">
+        <is>
+          <t>squaredawayvet.org
+gosquaredaway.com
+tsdr.uspto.gov/statusview/sn99277594
+uspto.report/TM/99252268</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1097,1698 +1598,1698 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
+    <row r="2" ht="44" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Numbered as on the shared naming page so a number is enough to refer to one. Twelve names carry a status; the other 88 are unsearched.</t>
+          <t>Numbered as on the shared naming page, so a number is enough to refer to one in conversation. Twelve carry a status; the other 88 are unsearched.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Status and findings</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="11" t="n">
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>Waypoint</t>
         </is>
       </c>
-      <c r="C5" s="13" t="inlineStr">
+      <c r="C5" s="23" t="inlineStr">
         <is>
           <t>Navigation and bearing</t>
         </is>
       </c>
-      <c r="D5" s="14" t="inlineStr">
-        <is>
-          <t>HIGH RISK: Sandboxx ships 'Waypoints', a military life app with TSP and PCS calculators: near-identical product and audience. Live Cl. 9 reg 5891296 covers downloadable guides and legal/business forms. waypoint.com is a debt collection agency. Waypoint Vets and DSPII Waypoint both operate in veteran services.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="11" t="n">
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>HIGH RISK: A near-identical military life app already ships to the same users.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
         <is>
           <t>Azimuth</t>
         </is>
       </c>
-      <c r="C6" s="13" t="inlineStr">
+      <c r="C6" s="23" t="inlineStr">
         <is>
           <t>Navigation and bearing</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>HIGH RISK: Trademark register is clear (all Azimuth regs in Cl. 9/36/41/42 are cancelled or abandoned) but the veteran space is colonized. 'Azimuth Check' is a US Army soldier well-being assessment; also GallantFew's Azimuth Check, the Azimuth Check Foundation, and Transition Azimuth Check (TrAC), a SOF military-to-civilian transition program. For a product positioned as 'not the VA', sharing a name with an Army assessment tool undercuts it. azimuth.org was a veteran resource nonprofit doing our exact job and now bounces to a parking lander: dormant prior use, not a clear field.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="58" customHeight="1">
-      <c r="A7" s="11" t="n">
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>HIGH RISK: The register is clear, which is the trap. The US Army already uses the phrase.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>Lodestar</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="C7" s="23" t="inlineStr">
         <is>
           <t>Navigation and bearing</t>
         </is>
       </c>
-      <c r="D7" s="14" t="inlineStr">
-        <is>
-          <t>CLEANEST VETERAN SPACE: Three targeted searches found no veteran nonprofit, transition program or military tool named Lodestar; only an internal employee resource group at a consulting firm. Ordinary problems remain: live Cl. 9 registration on the bare word (game studio, different field of use), live Cl. 36 for investment advisory, pending Cl. 41 and 42. lodestar.com is a national insurance claims administrator under Old Republic that rebranded onto it in 2026. The Lodestar name is heavily used across insurance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="58" customHeight="1">
-      <c r="A8" s="11" t="n">
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>CLEANEST VETERAN SPACE: No veteran nonprofit, transition program or military tool found using it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="15" t="inlineStr">
+      <c r="B8" s="24" t="inlineStr">
         <is>
           <t>Due North</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C8" s="23" t="inlineStr">
         <is>
           <t>Navigation and bearing</t>
         </is>
       </c>
-      <c r="D8" s="14" t="inlineStr">
-        <is>
-          <t>CLEANEST OVERALL: Zero veteran-space collisions found, the only such result among the twelve searched. Not clean, just cleanest: duenorth.com redirects to a PE-backed refrigeration manufacturer; SureWerx sells Due North(R) ice cleats using the registered symbol; live Cl. 45 registration for legal services; will be misheard as 'True North', an active US veterans nonprofit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="58" customHeight="1">
-      <c r="A9" s="11" t="n">
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>CLEANEST OVERALL: Zero veteran-space collisions, the only such result of the twelve.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="25" t="inlineStr">
         <is>
           <t>Trailhead</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="23" t="inlineStr">
         <is>
           <t>Navigation and bearing</t>
         </is>
       </c>
-      <c r="D9" s="14" t="inlineStr">
-        <is>
-          <t>RULE OUT: Salesforce owns TRAILHEAD (Reg. 5115199), LIVE, Classes 41 + 42, covering e-learning platforms and learning management systems. trailhead.com redirects to trailhead.salesforce.com. Salesforce also runs Trailhead Military for veterans and spouses. Project Trailhead is an existing veteran transition app.</t>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>RULE OUT: Salesforce owns the word in exactly our two classes, and runs a veteran programme under it.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="n">
+      <c r="A10" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="17" t="inlineStr">
+      <c r="B10" s="26" t="inlineStr">
         <is>
           <t>Bearing</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="C10" s="23" t="inlineStr">
         <is>
           <t>Navigation and bearing</t>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr"/>
+      <c r="D10" s="16" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="n">
+      <c r="A11" s="21" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="17" t="inlineStr">
+      <c r="B11" s="26" t="inlineStr">
         <is>
           <t>Vector</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C11" s="23" t="inlineStr">
         <is>
           <t>Navigation and bearing</t>
         </is>
       </c>
-      <c r="D11" s="14" t="inlineStr"/>
+      <c r="D11" s="16" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="n">
+      <c r="A12" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="17" t="inlineStr">
+      <c r="B12" s="26" t="inlineStr">
         <is>
           <t>Landfall</t>
         </is>
       </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="C12" s="23" t="inlineStr">
         <is>
           <t>Navigation and bearing</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
-    </row>
-    <row r="13" ht="58" customHeight="1">
-      <c r="A13" s="11" t="n">
+      <c r="D12" s="16" t="inlineStr"/>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="21" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B13" s="26" t="inlineStr">
         <is>
           <t>Sextant</t>
         </is>
       </c>
-      <c r="C13" s="13" t="inlineStr">
+      <c r="C13" s="23" t="inlineStr">
         <is>
           <t>Navigation and bearing</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
+      <c r="D13" s="16" t="inlineStr">
         <is>
           <t>CAUTION: Clean as a word, but the spelling trips content filters on some ad platforms.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="n">
+      <c r="A14" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="17" t="inlineStr">
+      <c r="B14" s="26" t="inlineStr">
         <is>
           <t>Waypost</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="C14" s="23" t="inlineStr">
         <is>
           <t>Navigation and bearing</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="D14" s="16" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="n">
+      <c r="A15" s="21" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="17" t="inlineStr">
+      <c r="B15" s="26" t="inlineStr">
         <is>
           <t>Compass Point</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
+      <c r="C15" s="23" t="inlineStr">
         <is>
           <t>Navigation and bearing</t>
         </is>
       </c>
-      <c r="D15" s="14" t="inlineStr"/>
+      <c r="D15" s="16" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="n">
+      <c r="A16" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="17" t="inlineStr">
+      <c r="B16" s="26" t="inlineStr">
         <is>
           <t>True Bearing</t>
         </is>
       </c>
-      <c r="C16" s="13" t="inlineStr">
+      <c r="C16" s="23" t="inlineStr">
         <is>
           <t>Navigation and bearing</t>
         </is>
       </c>
-      <c r="D16" s="14" t="inlineStr"/>
+      <c r="D16" s="16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="n">
+      <c r="A17" s="21" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="17" t="inlineStr">
+      <c r="B17" s="26" t="inlineStr">
         <is>
           <t>Northing</t>
         </is>
       </c>
-      <c r="C17" s="13" t="inlineStr">
+      <c r="C17" s="23" t="inlineStr">
         <is>
           <t>Navigation and bearing</t>
         </is>
       </c>
-      <c r="D17" s="14" t="inlineStr"/>
+      <c r="D17" s="16" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="n">
+      <c r="A18" s="21" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="17" t="inlineStr">
+      <c r="B18" s="26" t="inlineStr">
         <is>
           <t>Pilotage</t>
         </is>
       </c>
-      <c r="C18" s="13" t="inlineStr">
+      <c r="C18" s="23" t="inlineStr">
         <is>
           <t>Navigation and bearing</t>
         </is>
       </c>
-      <c r="D18" s="14" t="inlineStr"/>
-    </row>
-    <row r="19" ht="58" customHeight="1">
-      <c r="A19" s="11" t="n">
+      <c r="D18" s="16" t="inlineStr"/>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="21" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="12" t="inlineStr">
+      <c r="B19" s="22" t="inlineStr">
         <is>
           <t>Muster</t>
         </is>
       </c>
-      <c r="C19" s="13" t="inlineStr">
+      <c r="C19" s="23" t="inlineStr">
         <is>
           <t>Muster, formation, and the room</t>
         </is>
       </c>
-      <c r="D19" s="14" t="inlineStr">
-        <is>
-          <t>HIGH RISK: Echelon Front holds MUSTER (Reg. 5611610), LIVE and incontestable Feb 2025, Class 41 business education and training. Orion Talent launched Muster(TM) for veteran hiring on Veterans Day 2025. Adyton ships 'Mustr' to four service branches. Pending Cl. 9 filing for military social software. www.muster.com is advocacy SaaS.</t>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>HIGH RISK: Blocked by an incontestable Class 41 registration, and a veteran-hiring platform launched under it in 2025.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="n">
+      <c r="A20" s="21" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="17" t="inlineStr">
+      <c r="B20" s="26" t="inlineStr">
         <is>
           <t>Muster Point</t>
         </is>
       </c>
-      <c r="C20" s="13" t="inlineStr">
+      <c r="C20" s="23" t="inlineStr">
         <is>
           <t>Muster, formation, and the room</t>
         </is>
       </c>
-      <c r="D20" s="14" t="inlineStr"/>
-    </row>
-    <row r="21" ht="58" customHeight="1">
-      <c r="A21" s="11" t="n">
+      <c r="D20" s="16" t="inlineStr"/>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="21" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="25" t="inlineStr">
         <is>
           <t>Rally Point</t>
         </is>
       </c>
-      <c r="C21" s="13" t="inlineStr">
+      <c r="C21" s="23" t="inlineStr">
         <is>
           <t>Muster, formation, and the room</t>
         </is>
       </c>
-      <c r="D21" s="14" t="inlineStr">
-        <is>
-          <t>RULE OUT: RallyPoint Networks holds 5 live registrations (Cl. 35/38/41/45), incontestable. Reg. 4730603 covers websites with employment listings and training info for military personnel. Counsel: Latham &amp; Watkins. Five other veteran orgs use the name. Site down since ~Mar 2026 but marks run for years.</t>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>RULE OUT: Five live incontestable registrations describing our product in trademark language.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="n">
+      <c r="A22" s="21" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="17" t="inlineStr">
+      <c r="B22" s="26" t="inlineStr">
         <is>
           <t>Formation</t>
         </is>
       </c>
-      <c r="C22" s="13" t="inlineStr">
+      <c r="C22" s="23" t="inlineStr">
         <is>
           <t>Muster, formation, and the room</t>
         </is>
       </c>
-      <c r="D22" s="14" t="inlineStr"/>
+      <c r="D22" s="16" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="n">
+      <c r="A23" s="21" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="17" t="inlineStr">
+      <c r="B23" s="26" t="inlineStr">
         <is>
           <t>Next Formation</t>
         </is>
       </c>
-      <c r="C23" s="13" t="inlineStr">
+      <c r="C23" s="23" t="inlineStr">
         <is>
           <t>Muster, formation, and the room</t>
         </is>
       </c>
-      <c r="D23" s="14" t="inlineStr"/>
+      <c r="D23" s="16" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="11" t="n">
+      <c r="A24" s="21" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="17" t="inlineStr">
+      <c r="B24" s="26" t="inlineStr">
         <is>
           <t>Guidon</t>
         </is>
       </c>
-      <c r="C24" s="13" t="inlineStr">
+      <c r="C24" s="23" t="inlineStr">
         <is>
           <t>Muster, formation, and the room</t>
         </is>
       </c>
-      <c r="D24" s="14" t="inlineStr"/>
+      <c r="D24" s="16" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="n">
+      <c r="A25" s="21" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="17" t="inlineStr">
+      <c r="B25" s="26" t="inlineStr">
         <is>
           <t>Echelon</t>
         </is>
       </c>
-      <c r="C25" s="13" t="inlineStr">
+      <c r="C25" s="23" t="inlineStr">
         <is>
           <t>Muster, formation, and the room</t>
         </is>
       </c>
-      <c r="D25" s="14" t="inlineStr"/>
+      <c r="D25" s="16" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="11" t="n">
+      <c r="A26" s="21" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="17" t="inlineStr">
+      <c r="B26" s="26" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C26" s="13" t="inlineStr">
+      <c r="C26" s="23" t="inlineStr">
         <is>
           <t>Muster, formation, and the room</t>
         </is>
       </c>
-      <c r="D26" s="14" t="inlineStr"/>
+      <c r="D26" s="16" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="n">
+      <c r="A27" s="21" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="17" t="inlineStr">
+      <c r="B27" s="26" t="inlineStr">
         <is>
           <t>Assembly</t>
         </is>
       </c>
-      <c r="C27" s="13" t="inlineStr">
+      <c r="C27" s="23" t="inlineStr">
         <is>
           <t>Muster, formation, and the room</t>
         </is>
       </c>
-      <c r="D27" s="14" t="inlineStr"/>
+      <c r="D27" s="16" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="11" t="n">
+      <c r="A28" s="21" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="17" t="inlineStr">
+      <c r="B28" s="26" t="inlineStr">
         <is>
           <t>Quorum</t>
         </is>
       </c>
-      <c r="C28" s="13" t="inlineStr">
+      <c r="C28" s="23" t="inlineStr">
         <is>
           <t>Muster, formation, and the room</t>
         </is>
       </c>
-      <c r="D28" s="14" t="inlineStr"/>
+      <c r="D28" s="16" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="11" t="n">
+      <c r="A29" s="21" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="17" t="inlineStr">
+      <c r="B29" s="26" t="inlineStr">
         <is>
           <t>The Table</t>
         </is>
       </c>
-      <c r="C29" s="13" t="inlineStr">
+      <c r="C29" s="23" t="inlineStr">
         <is>
           <t>Muster, formation, and the room</t>
         </is>
       </c>
-      <c r="D29" s="14" t="inlineStr"/>
+      <c r="D29" s="16" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="n">
+      <c r="A30" s="21" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="17" t="inlineStr">
+      <c r="B30" s="26" t="inlineStr">
         <is>
           <t>Roundtable</t>
         </is>
       </c>
-      <c r="C30" s="13" t="inlineStr">
+      <c r="C30" s="23" t="inlineStr">
         <is>
           <t>Muster, formation, and the room</t>
         </is>
       </c>
-      <c r="D30" s="14" t="inlineStr"/>
+      <c r="D30" s="16" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="11" t="n">
+      <c r="A31" s="21" t="n">
         <v>27</v>
       </c>
-      <c r="B31" s="17" t="inlineStr">
+      <c r="B31" s="26" t="inlineStr">
         <is>
           <t>Huddle</t>
         </is>
       </c>
-      <c r="C31" s="13" t="inlineStr">
+      <c r="C31" s="23" t="inlineStr">
         <is>
           <t>Muster, formation, and the room</t>
         </is>
       </c>
-      <c r="D31" s="14" t="inlineStr"/>
+      <c r="D31" s="16" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="11" t="n">
+      <c r="A32" s="21" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="17" t="inlineStr">
+      <c r="B32" s="26" t="inlineStr">
         <is>
           <t>Circle Up</t>
         </is>
       </c>
-      <c r="C32" s="13" t="inlineStr">
+      <c r="C32" s="23" t="inlineStr">
         <is>
           <t>Muster, formation, and the room</t>
         </is>
       </c>
-      <c r="D32" s="14" t="inlineStr"/>
-    </row>
-    <row r="33" ht="58" customHeight="1">
-      <c r="A33" s="11" t="n">
+      <c r="D32" s="16" t="inlineStr"/>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="21" t="n">
         <v>29</v>
       </c>
-      <c r="B33" s="12" t="inlineStr">
+      <c r="B33" s="22" t="inlineStr">
         <is>
           <t>Reveille</t>
         </is>
       </c>
-      <c r="C33" s="13" t="inlineStr">
+      <c r="C33" s="23" t="inlineStr">
         <is>
           <t>Calls, signals, first light</t>
         </is>
       </c>
-      <c r="D33" s="14" t="inlineStr">
-        <is>
-          <t>HIGH RISK: Reveille and Retreat Project holds Reg. 8164652, LIVE, Class 41, education for female veterans and service members. Reveille Foundation runs veteran housing and employment with DOL/VA ties. Reveille Grounds is a veteran coworking hub. Texas A&amp;M mascot claim is a separate overhang. reveille.com held since 1991.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="58" customHeight="1">
-      <c r="A34" s="11" t="n">
+      <c r="D33" s="16" t="inlineStr">
+        <is>
+          <t>HIGH RISK: Three veteran organisations use it, one holding a live registration in our class.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="21" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="18" t="inlineStr">
+      <c r="B34" s="27" t="inlineStr">
         <is>
           <t>First Light</t>
         </is>
       </c>
-      <c r="C34" s="13" t="inlineStr">
+      <c r="C34" s="23" t="inlineStr">
         <is>
           <t>Calls, signals, first light</t>
         </is>
       </c>
-      <c r="D34" s="14" t="inlineStr">
-        <is>
-          <t>USABLE, WITH DRAG: Crowded but diffuse: nobody owns it in veteran benefits or career planning. firstlight.com is a stock photography company; firstlight.net is a regional fiber telecom. Class 36 has four live registrations including FirstLight Federal Credit Union, which serves Fort Bliss and runs a Veterans Benefits Banking Program. Cl. 42 has two live SaaS registrations, Cl. 9 one active. A permanent disambiguation tax rather than a single fatal blocker.</t>
+      <c r="D34" s="16" t="inlineStr">
+        <is>
+          <t>USABLE, WITH DRAG: Crowded but diffusely: nobody owns it in veteran benefits or career planning.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="11" t="n">
+      <c r="A35" s="21" t="n">
         <v>31</v>
       </c>
-      <c r="B35" s="17" t="inlineStr">
+      <c r="B35" s="26" t="inlineStr">
         <is>
           <t>Daybreak</t>
         </is>
       </c>
-      <c r="C35" s="13" t="inlineStr">
+      <c r="C35" s="23" t="inlineStr">
         <is>
           <t>Calls, signals, first light</t>
         </is>
       </c>
-      <c r="D35" s="14" t="inlineStr"/>
+      <c r="D35" s="16" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="11" t="n">
+      <c r="A36" s="21" t="n">
         <v>32</v>
       </c>
-      <c r="B36" s="17" t="inlineStr">
+      <c r="B36" s="26" t="inlineStr">
         <is>
           <t>Stand To</t>
         </is>
       </c>
-      <c r="C36" s="13" t="inlineStr">
+      <c r="C36" s="23" t="inlineStr">
         <is>
           <t>Calls, signals, first light</t>
         </is>
       </c>
-      <c r="D36" s="14" t="inlineStr"/>
+      <c r="D36" s="16" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="11" t="n">
+      <c r="A37" s="21" t="n">
         <v>33</v>
       </c>
-      <c r="B37" s="17" t="inlineStr">
+      <c r="B37" s="26" t="inlineStr">
         <is>
           <t>Cadence</t>
         </is>
       </c>
-      <c r="C37" s="13" t="inlineStr">
+      <c r="C37" s="23" t="inlineStr">
         <is>
           <t>Calls, signals, first light</t>
         </is>
       </c>
-      <c r="D37" s="14" t="inlineStr"/>
+      <c r="D37" s="16" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="11" t="n">
+      <c r="A38" s="21" t="n">
         <v>34</v>
       </c>
-      <c r="B38" s="17" t="inlineStr">
+      <c r="B38" s="26" t="inlineStr">
         <is>
           <t>Colors</t>
         </is>
       </c>
-      <c r="C38" s="13" t="inlineStr">
+      <c r="C38" s="23" t="inlineStr">
         <is>
           <t>Calls, signals, first light</t>
         </is>
       </c>
-      <c r="D38" s="14" t="inlineStr"/>
+      <c r="D38" s="16" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="11" t="n">
+      <c r="A39" s="21" t="n">
         <v>35</v>
       </c>
-      <c r="B39" s="17" t="inlineStr">
+      <c r="B39" s="26" t="inlineStr">
         <is>
           <t>Beacon</t>
         </is>
       </c>
-      <c r="C39" s="13" t="inlineStr">
+      <c r="C39" s="23" t="inlineStr">
         <is>
           <t>Calls, signals, first light</t>
         </is>
       </c>
-      <c r="D39" s="14" t="inlineStr"/>
-    </row>
-    <row r="40" ht="58" customHeight="1">
-      <c r="A40" s="11" t="n">
+      <c r="D39" s="16" t="inlineStr"/>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="21" t="n">
         <v>36</v>
       </c>
-      <c r="B40" s="16" t="inlineStr">
+      <c r="B40" s="26" t="inlineStr">
         <is>
           <t>Signal</t>
         </is>
       </c>
-      <c r="C40" s="13" t="inlineStr">
+      <c r="C40" s="23" t="inlineStr">
         <is>
           <t>Calls, signals, first light</t>
         </is>
       </c>
-      <c r="D40" s="14" t="inlineStr">
+      <c r="D40" s="16" t="inlineStr">
         <is>
           <t>KNOWN CONFLICT: Signal is a major encrypted-messaging brand.</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="11" t="n">
+      <c r="A41" s="21" t="n">
         <v>37</v>
       </c>
-      <c r="B41" s="17" t="inlineStr">
+      <c r="B41" s="26" t="inlineStr">
         <is>
           <t>Semaphore</t>
         </is>
       </c>
-      <c r="C41" s="13" t="inlineStr">
+      <c r="C41" s="23" t="inlineStr">
         <is>
           <t>Calls, signals, first light</t>
         </is>
       </c>
-      <c r="D41" s="14" t="inlineStr"/>
+      <c r="D41" s="16" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="11" t="n">
+      <c r="A42" s="21" t="n">
         <v>38</v>
       </c>
-      <c r="B42" s="17" t="inlineStr">
+      <c r="B42" s="26" t="inlineStr">
         <is>
           <t>Watchfire</t>
         </is>
       </c>
-      <c r="C42" s="13" t="inlineStr">
+      <c r="C42" s="23" t="inlineStr">
         <is>
           <t>Calls, signals, first light</t>
         </is>
       </c>
-      <c r="D42" s="14" t="inlineStr"/>
+      <c r="D42" s="16" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="11" t="n">
+      <c r="A43" s="21" t="n">
         <v>39</v>
       </c>
-      <c r="B43" s="17" t="inlineStr">
+      <c r="B43" s="26" t="inlineStr">
         <is>
           <t>Dawn Patrol</t>
         </is>
       </c>
-      <c r="C43" s="13" t="inlineStr">
+      <c r="C43" s="23" t="inlineStr">
         <is>
           <t>Calls, signals, first light</t>
         </is>
       </c>
-      <c r="D43" s="14" t="inlineStr"/>
+      <c r="D43" s="16" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="11" t="n">
+      <c r="A44" s="21" t="n">
         <v>40</v>
       </c>
-      <c r="B44" s="17" t="inlineStr">
+      <c r="B44" s="26" t="inlineStr">
         <is>
           <t>Sunup</t>
         </is>
       </c>
-      <c r="C44" s="13" t="inlineStr">
+      <c r="C44" s="23" t="inlineStr">
         <is>
           <t>Calls, signals, first light</t>
         </is>
       </c>
-      <c r="D44" s="14" t="inlineStr"/>
-    </row>
-    <row r="45" ht="58" customHeight="1">
-      <c r="A45" s="11" t="n">
+      <c r="D44" s="16" t="inlineStr"/>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="21" t="n">
         <v>41</v>
       </c>
-      <c r="B45" s="18" t="inlineStr">
+      <c r="B45" s="27" t="inlineStr">
         <is>
           <t>After Action</t>
         </is>
       </c>
-      <c r="C45" s="13" t="inlineStr">
+      <c r="C45" s="23" t="inlineStr">
         <is>
           <t>The brief and the debrief</t>
         </is>
       </c>
-      <c r="D45" s="14" t="inlineStr">
-        <is>
-          <t>USABLE, WITH DRAG: No live registered mark found blocking Cl. 9/35/36/41/42/45; the one veteran Cl. 41 filing was abandoned 2016. Cleanest trademark result of the eight. Drag: 'after action review' is military doctrine so it is weakly distinctive; 4+ veteran media brands use it including a PBS series; afteraction.com does not resolve; the old After Action Network lost its .org to an adult-content site.</t>
+      <c r="D45" s="16" t="inlineStr">
+        <is>
+          <t>USABLE, WITH DRAG: Cleanest trademark result: no live registered mark found blocking our classes.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="11" t="n">
+      <c r="A46" s="21" t="n">
         <v>42</v>
       </c>
-      <c r="B46" s="17" t="inlineStr">
+      <c r="B46" s="26" t="inlineStr">
         <is>
           <t>Debrief</t>
         </is>
       </c>
-      <c r="C46" s="13" t="inlineStr">
+      <c r="C46" s="23" t="inlineStr">
         <is>
           <t>The brief and the debrief</t>
         </is>
       </c>
-      <c r="D46" s="14" t="inlineStr"/>
+      <c r="D46" s="16" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="11" t="n">
+      <c r="A47" s="21" t="n">
         <v>43</v>
       </c>
-      <c r="B47" s="17" t="inlineStr">
+      <c r="B47" s="26" t="inlineStr">
         <is>
           <t>The Brief</t>
         </is>
       </c>
-      <c r="C47" s="13" t="inlineStr">
+      <c r="C47" s="23" t="inlineStr">
         <is>
           <t>The brief and the debrief</t>
         </is>
       </c>
-      <c r="D47" s="14" t="inlineStr"/>
+      <c r="D47" s="16" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="11" t="n">
+      <c r="A48" s="21" t="n">
         <v>44</v>
       </c>
-      <c r="B48" s="17" t="inlineStr">
+      <c r="B48" s="26" t="inlineStr">
         <is>
           <t>Sitrep</t>
         </is>
       </c>
-      <c r="C48" s="13" t="inlineStr">
+      <c r="C48" s="23" t="inlineStr">
         <is>
           <t>The brief and the debrief</t>
         </is>
       </c>
-      <c r="D48" s="14" t="inlineStr"/>
+      <c r="D48" s="16" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="11" t="n">
+      <c r="A49" s="21" t="n">
         <v>45</v>
       </c>
-      <c r="B49" s="17" t="inlineStr">
+      <c r="B49" s="26" t="inlineStr">
         <is>
           <t>Field Manual</t>
         </is>
       </c>
-      <c r="C49" s="13" t="inlineStr">
+      <c r="C49" s="23" t="inlineStr">
         <is>
           <t>The brief and the debrief</t>
         </is>
       </c>
-      <c r="D49" s="14" t="inlineStr"/>
+      <c r="D49" s="16" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="11" t="n">
+      <c r="A50" s="21" t="n">
         <v>46</v>
       </c>
-      <c r="B50" s="17" t="inlineStr">
+      <c r="B50" s="26" t="inlineStr">
         <is>
           <t>The Manual</t>
         </is>
       </c>
-      <c r="C50" s="13" t="inlineStr">
+      <c r="C50" s="23" t="inlineStr">
         <is>
           <t>The brief and the debrief</t>
         </is>
       </c>
-      <c r="D50" s="14" t="inlineStr"/>
+      <c r="D50" s="16" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="11" t="n">
+      <c r="A51" s="21" t="n">
         <v>47</v>
       </c>
-      <c r="B51" s="17" t="inlineStr">
+      <c r="B51" s="26" t="inlineStr">
         <is>
           <t>Standing Orders</t>
         </is>
       </c>
-      <c r="C51" s="13" t="inlineStr">
+      <c r="C51" s="23" t="inlineStr">
         <is>
           <t>The brief and the debrief</t>
         </is>
       </c>
-      <c r="D51" s="14" t="inlineStr"/>
+      <c r="D51" s="16" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="11" t="n">
+      <c r="A52" s="21" t="n">
         <v>48</v>
       </c>
-      <c r="B52" s="17" t="inlineStr">
+      <c r="B52" s="26" t="inlineStr">
         <is>
           <t>Order of March</t>
         </is>
       </c>
-      <c r="C52" s="13" t="inlineStr">
+      <c r="C52" s="23" t="inlineStr">
         <is>
           <t>The brief and the debrief</t>
         </is>
       </c>
-      <c r="D52" s="14" t="inlineStr"/>
+      <c r="D52" s="16" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="11" t="n">
+      <c r="A53" s="21" t="n">
         <v>49</v>
       </c>
-      <c r="B53" s="17" t="inlineStr">
+      <c r="B53" s="26" t="inlineStr">
         <is>
           <t>Warning Order</t>
         </is>
       </c>
-      <c r="C53" s="13" t="inlineStr">
+      <c r="C53" s="23" t="inlineStr">
         <is>
           <t>The brief and the debrief</t>
         </is>
       </c>
-      <c r="D53" s="14" t="inlineStr"/>
+      <c r="D53" s="16" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="11" t="n">
+      <c r="A54" s="21" t="n">
         <v>50</v>
       </c>
-      <c r="B54" s="17" t="inlineStr">
+      <c r="B54" s="26" t="inlineStr">
         <is>
           <t>Checklist</t>
         </is>
       </c>
-      <c r="C54" s="13" t="inlineStr">
+      <c r="C54" s="23" t="inlineStr">
         <is>
           <t>The brief and the debrief</t>
         </is>
       </c>
-      <c r="D54" s="14" t="inlineStr"/>
+      <c r="D54" s="16" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="11" t="n">
+      <c r="A55" s="21" t="n">
         <v>51</v>
       </c>
-      <c r="B55" s="17" t="inlineStr">
+      <c r="B55" s="26" t="inlineStr">
         <is>
           <t>Ledger</t>
         </is>
       </c>
-      <c r="C55" s="13" t="inlineStr">
+      <c r="C55" s="23" t="inlineStr">
         <is>
           <t>The brief and the debrief</t>
         </is>
       </c>
-      <c r="D55" s="14" t="inlineStr"/>
+      <c r="D55" s="16" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="11" t="n">
+      <c r="A56" s="21" t="n">
         <v>52</v>
       </c>
-      <c r="B56" s="17" t="inlineStr">
+      <c r="B56" s="26" t="inlineStr">
         <is>
           <t>Dossier</t>
         </is>
       </c>
-      <c r="C56" s="13" t="inlineStr">
+      <c r="C56" s="23" t="inlineStr">
         <is>
           <t>The brief and the debrief</t>
         </is>
       </c>
-      <c r="D56" s="14" t="inlineStr"/>
-    </row>
-    <row r="57" ht="58" customHeight="1">
-      <c r="A57" s="11" t="n">
+      <c r="D56" s="16" t="inlineStr"/>
+    </row>
+    <row r="57" ht="30" customHeight="1">
+      <c r="A57" s="21" t="n">
         <v>53</v>
       </c>
-      <c r="B57" s="18" t="inlineStr">
+      <c r="B57" s="27" t="inlineStr">
         <is>
           <t>Earned</t>
         </is>
       </c>
-      <c r="C57" s="13" t="inlineStr">
+      <c r="C57" s="23" t="inlineStr">
         <is>
           <t>Earned, not given</t>
         </is>
       </c>
-      <c r="D57" s="14" t="inlineStr">
-        <is>
-          <t>USABLE, WITH DRAG: No plain-word registration found in our classes and no veteran-space entity uses it. But earned.com belongs to Earned Wealth ($200M raised, $3.9B AUM, consumer finance app, filing new marks in 2026). 'Earned benefits' is standard VA vocabulary, so organic search would be severely handicapped.</t>
+      <c r="D57" s="16" t="inlineStr">
+        <is>
+          <t>USABLE, WITH DRAG: No blocking registration and no veteran-space entity, but the .com and search are problems.</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="11" t="n">
+      <c r="A58" s="21" t="n">
         <v>54</v>
       </c>
-      <c r="B58" s="17" t="inlineStr">
+      <c r="B58" s="26" t="inlineStr">
         <is>
           <t>Well Earned</t>
         </is>
       </c>
-      <c r="C58" s="13" t="inlineStr">
+      <c r="C58" s="23" t="inlineStr">
         <is>
           <t>Earned, not given</t>
         </is>
       </c>
-      <c r="D58" s="14" t="inlineStr"/>
+      <c r="D58" s="16" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="11" t="n">
+      <c r="A59" s="21" t="n">
         <v>55</v>
       </c>
-      <c r="B59" s="17" t="inlineStr">
+      <c r="B59" s="26" t="inlineStr">
         <is>
           <t>Hard Earned</t>
         </is>
       </c>
-      <c r="C59" s="13" t="inlineStr">
+      <c r="C59" s="23" t="inlineStr">
         <is>
           <t>Earned, not given</t>
         </is>
       </c>
-      <c r="D59" s="14" t="inlineStr"/>
+      <c r="D59" s="16" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="11" t="n">
+      <c r="A60" s="21" t="n">
         <v>56</v>
       </c>
-      <c r="B60" s="17" t="inlineStr">
+      <c r="B60" s="26" t="inlineStr">
         <is>
           <t>By Right</t>
         </is>
       </c>
-      <c r="C60" s="13" t="inlineStr">
+      <c r="C60" s="23" t="inlineStr">
         <is>
           <t>Earned, not given</t>
         </is>
       </c>
-      <c r="D60" s="14" t="inlineStr"/>
+      <c r="D60" s="16" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="11" t="n">
+      <c r="A61" s="21" t="n">
         <v>57</v>
       </c>
-      <c r="B61" s="17" t="inlineStr">
+      <c r="B61" s="26" t="inlineStr">
         <is>
           <t>Rightful</t>
         </is>
       </c>
-      <c r="C61" s="13" t="inlineStr">
+      <c r="C61" s="23" t="inlineStr">
         <is>
           <t>Earned, not given</t>
         </is>
       </c>
-      <c r="D61" s="14" t="inlineStr"/>
+      <c r="D61" s="16" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="11" t="n">
+      <c r="A62" s="21" t="n">
         <v>58</v>
       </c>
-      <c r="B62" s="17" t="inlineStr">
+      <c r="B62" s="26" t="inlineStr">
         <is>
           <t>Merit</t>
         </is>
       </c>
-      <c r="C62" s="13" t="inlineStr">
+      <c r="C62" s="23" t="inlineStr">
         <is>
           <t>Earned, not given</t>
         </is>
       </c>
-      <c r="D62" s="14" t="inlineStr"/>
+      <c r="D62" s="16" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="11" t="n">
+      <c r="A63" s="21" t="n">
         <v>59</v>
       </c>
-      <c r="B63" s="17" t="inlineStr">
+      <c r="B63" s="26" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="C63" s="13" t="inlineStr">
+      <c r="C63" s="23" t="inlineStr">
         <is>
           <t>Earned, not given</t>
         </is>
       </c>
-      <c r="D63" s="14" t="inlineStr"/>
+      <c r="D63" s="16" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="11" t="n">
+      <c r="A64" s="21" t="n">
         <v>60</v>
       </c>
-      <c r="B64" s="17" t="inlineStr">
+      <c r="B64" s="26" t="inlineStr">
         <is>
           <t>Full Benefit</t>
         </is>
       </c>
-      <c r="C64" s="13" t="inlineStr">
+      <c r="C64" s="23" t="inlineStr">
         <is>
           <t>Earned, not given</t>
         </is>
       </c>
-      <c r="D64" s="14" t="inlineStr"/>
+      <c r="D64" s="16" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="11" t="n">
+      <c r="A65" s="21" t="n">
         <v>61</v>
       </c>
-      <c r="B65" s="17" t="inlineStr">
+      <c r="B65" s="26" t="inlineStr">
         <is>
           <t>Every Benefit</t>
         </is>
       </c>
-      <c r="C65" s="13" t="inlineStr">
+      <c r="C65" s="23" t="inlineStr">
         <is>
           <t>Earned, not given</t>
         </is>
       </c>
-      <c r="D65" s="14" t="inlineStr"/>
-    </row>
-    <row r="66" ht="58" customHeight="1">
-      <c r="A66" s="11" t="n">
+      <c r="D65" s="16" t="inlineStr"/>
+    </row>
+    <row r="66" ht="30" customHeight="1">
+      <c r="A66" s="21" t="n">
         <v>62</v>
       </c>
-      <c r="B66" s="16" t="inlineStr">
+      <c r="B66" s="25" t="inlineStr">
         <is>
           <t>Squared Away</t>
         </is>
       </c>
-      <c r="C66" s="13" t="inlineStr">
+      <c r="C66" s="23" t="inlineStr">
         <is>
           <t>Earned, not given</t>
         </is>
       </c>
-      <c r="D66" s="14" t="inlineStr">
-        <is>
-          <t>RULE OUT: squaredawayvet.org is live and is our product: 'your personal Hub for Veteran resources and documents', with pages for Documents, Education Benefits, Service Connection, Communities and Colleges. First Command (68-year-old military financial firm) holds a live Cl. 36 registration and markets 'Get Your Finances Squared Away' to service members. The military-spouse staffing firm Squared Away made the Inc. 5000. Two more applications in prosecution: Cl. 9 for software organizing military personnel, and a multi-class veteran app. Every class we occupy has a live or pending mark, and the phrase is ordinary military slang so distinctiveness is unreachable.</t>
+      <c r="D66" s="16" t="inlineStr">
+        <is>
+          <t>RULE OUT: Someone is already running this exact product under this exact name.</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="11" t="n">
+      <c r="A67" s="21" t="n">
         <v>63</v>
       </c>
-      <c r="B67" s="17" t="inlineStr">
+      <c r="B67" s="26" t="inlineStr">
         <is>
           <t>Accounted For</t>
         </is>
       </c>
-      <c r="C67" s="13" t="inlineStr">
+      <c r="C67" s="23" t="inlineStr">
         <is>
           <t>Earned, not given</t>
         </is>
       </c>
-      <c r="D67" s="14" t="inlineStr"/>
+      <c r="D67" s="16" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="11" t="n">
+      <c r="A68" s="21" t="n">
         <v>64</v>
       </c>
-      <c r="B68" s="17" t="inlineStr">
+      <c r="B68" s="26" t="inlineStr">
         <is>
           <t>In Full</t>
         </is>
       </c>
-      <c r="C68" s="13" t="inlineStr">
+      <c r="C68" s="23" t="inlineStr">
         <is>
           <t>Earned, not given</t>
         </is>
       </c>
-      <c r="D68" s="14" t="inlineStr"/>
+      <c r="D68" s="16" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="11" t="n">
+      <c r="A69" s="21" t="n">
         <v>65</v>
       </c>
-      <c r="B69" s="17" t="inlineStr">
+      <c r="B69" s="26" t="inlineStr">
         <is>
           <t>Next Chapter</t>
         </is>
       </c>
-      <c r="C69" s="13" t="inlineStr">
+      <c r="C69" s="23" t="inlineStr">
         <is>
           <t>The next chapter</t>
         </is>
       </c>
-      <c r="D69" s="14" t="inlineStr"/>
+      <c r="D69" s="16" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="11" t="n">
+      <c r="A70" s="21" t="n">
         <v>66</v>
       </c>
-      <c r="B70" s="17" t="inlineStr">
+      <c r="B70" s="26" t="inlineStr">
         <is>
           <t>Chapter Two</t>
         </is>
       </c>
-      <c r="C70" s="13" t="inlineStr">
+      <c r="C70" s="23" t="inlineStr">
         <is>
           <t>The next chapter</t>
         </is>
       </c>
-      <c r="D70" s="14" t="inlineStr"/>
+      <c r="D70" s="16" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="11" t="n">
+      <c r="A71" s="21" t="n">
         <v>67</v>
       </c>
-      <c r="B71" s="17" t="inlineStr">
+      <c r="B71" s="26" t="inlineStr">
         <is>
           <t>Second Service</t>
         </is>
       </c>
-      <c r="C71" s="13" t="inlineStr">
+      <c r="C71" s="23" t="inlineStr">
         <is>
           <t>The next chapter</t>
         </is>
       </c>
-      <c r="D71" s="14" t="inlineStr"/>
+      <c r="D71" s="16" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="11" t="n">
+      <c r="A72" s="21" t="n">
         <v>68</v>
       </c>
-      <c r="B72" s="17" t="inlineStr">
+      <c r="B72" s="26" t="inlineStr">
         <is>
           <t>Still Serving</t>
         </is>
       </c>
-      <c r="C72" s="13" t="inlineStr">
+      <c r="C72" s="23" t="inlineStr">
         <is>
           <t>The next chapter</t>
         </is>
       </c>
-      <c r="D72" s="14" t="inlineStr"/>
+      <c r="D72" s="16" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" s="11" t="n">
+      <c r="A73" s="21" t="n">
         <v>69</v>
       </c>
-      <c r="B73" s="17" t="inlineStr">
+      <c r="B73" s="26" t="inlineStr">
         <is>
           <t>Out of Uniform</t>
         </is>
       </c>
-      <c r="C73" s="13" t="inlineStr">
+      <c r="C73" s="23" t="inlineStr">
         <is>
           <t>The next chapter</t>
         </is>
       </c>
-      <c r="D73" s="14" t="inlineStr"/>
+      <c r="D73" s="16" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" s="11" t="n">
+      <c r="A74" s="21" t="n">
         <v>70</v>
       </c>
-      <c r="B74" s="17" t="inlineStr">
+      <c r="B74" s="26" t="inlineStr">
         <is>
           <t>Next Mission</t>
         </is>
       </c>
-      <c r="C74" s="13" t="inlineStr">
+      <c r="C74" s="23" t="inlineStr">
         <is>
           <t>The next chapter</t>
         </is>
       </c>
-      <c r="D74" s="14" t="inlineStr"/>
+      <c r="D74" s="16" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" s="11" t="n">
+      <c r="A75" s="21" t="n">
         <v>71</v>
       </c>
-      <c r="B75" s="17" t="inlineStr">
+      <c r="B75" s="26" t="inlineStr">
         <is>
           <t>Homeward</t>
         </is>
       </c>
-      <c r="C75" s="13" t="inlineStr">
+      <c r="C75" s="23" t="inlineStr">
         <is>
           <t>The next chapter</t>
         </is>
       </c>
-      <c r="D75" s="14" t="inlineStr"/>
+      <c r="D75" s="16" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" s="11" t="n">
+      <c r="A76" s="21" t="n">
         <v>72</v>
       </c>
-      <c r="B76" s="17" t="inlineStr">
+      <c r="B76" s="26" t="inlineStr">
         <is>
           <t>Homefront</t>
         </is>
       </c>
-      <c r="C76" s="13" t="inlineStr">
+      <c r="C76" s="23" t="inlineStr">
         <is>
           <t>The next chapter</t>
         </is>
       </c>
-      <c r="D76" s="14" t="inlineStr"/>
+      <c r="D76" s="16" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" s="11" t="n">
+      <c r="A77" s="21" t="n">
         <v>73</v>
       </c>
-      <c r="B77" s="17" t="inlineStr">
+      <c r="B77" s="26" t="inlineStr">
         <is>
           <t>Landing</t>
         </is>
       </c>
-      <c r="C77" s="13" t="inlineStr">
+      <c r="C77" s="23" t="inlineStr">
         <is>
           <t>The next chapter</t>
         </is>
       </c>
-      <c r="D77" s="14" t="inlineStr"/>
+      <c r="D77" s="16" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" s="11" t="n">
+      <c r="A78" s="21" t="n">
         <v>74</v>
       </c>
-      <c r="B78" s="17" t="inlineStr">
+      <c r="B78" s="26" t="inlineStr">
         <is>
           <t>Soft Landing</t>
         </is>
       </c>
-      <c r="C78" s="13" t="inlineStr">
+      <c r="C78" s="23" t="inlineStr">
         <is>
           <t>The next chapter</t>
         </is>
       </c>
-      <c r="D78" s="14" t="inlineStr"/>
+      <c r="D78" s="16" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" s="11" t="n">
+      <c r="A79" s="21" t="n">
         <v>75</v>
       </c>
-      <c r="B79" s="17" t="inlineStr">
+      <c r="B79" s="26" t="inlineStr">
         <is>
           <t>Crossing</t>
         </is>
       </c>
-      <c r="C79" s="13" t="inlineStr">
+      <c r="C79" s="23" t="inlineStr">
         <is>
           <t>The next chapter</t>
         </is>
       </c>
-      <c r="D79" s="14" t="inlineStr"/>
+      <c r="D79" s="16" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" s="11" t="n">
+      <c r="A80" s="21" t="n">
         <v>76</v>
       </c>
-      <c r="B80" s="17" t="inlineStr">
+      <c r="B80" s="26" t="inlineStr">
         <is>
           <t>Threshold</t>
         </is>
       </c>
-      <c r="C80" s="13" t="inlineStr">
+      <c r="C80" s="23" t="inlineStr">
         <is>
           <t>The next chapter</t>
         </is>
       </c>
-      <c r="D80" s="14" t="inlineStr"/>
+      <c r="D80" s="16" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" s="11" t="n">
+      <c r="A81" s="21" t="n">
         <v>77</v>
       </c>
-      <c r="B81" s="17" t="inlineStr">
+      <c r="B81" s="26" t="inlineStr">
         <is>
           <t>Horizon</t>
         </is>
       </c>
-      <c r="C81" s="13" t="inlineStr">
+      <c r="C81" s="23" t="inlineStr">
         <is>
           <t>The next chapter</t>
         </is>
       </c>
-      <c r="D81" s="14" t="inlineStr"/>
+      <c r="D81" s="16" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" s="11" t="n">
+      <c r="A82" s="21" t="n">
         <v>78</v>
       </c>
-      <c r="B82" s="17" t="inlineStr">
+      <c r="B82" s="26" t="inlineStr">
         <is>
           <t>Afterburner</t>
         </is>
       </c>
-      <c r="C82" s="13" t="inlineStr">
+      <c r="C82" s="23" t="inlineStr">
         <is>
           <t>The next chapter</t>
         </is>
       </c>
-      <c r="D82" s="14" t="inlineStr"/>
+      <c r="D82" s="16" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="A83" s="11" t="n">
+      <c r="A83" s="21" t="n">
         <v>79</v>
       </c>
-      <c r="B83" s="17" t="inlineStr">
+      <c r="B83" s="26" t="inlineStr">
         <is>
           <t>Ninety</t>
         </is>
       </c>
-      <c r="C83" s="13" t="inlineStr">
+      <c r="C83" s="23" t="inlineStr">
         <is>
           <t>The plan and the ninety days</t>
         </is>
       </c>
-      <c r="D83" s="14" t="inlineStr"/>
+      <c r="D83" s="16" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" s="11" t="n">
+      <c r="A84" s="21" t="n">
         <v>80</v>
       </c>
-      <c r="B84" s="17" t="inlineStr">
+      <c r="B84" s="26" t="inlineStr">
         <is>
           <t>First Ninety</t>
         </is>
       </c>
-      <c r="C84" s="13" t="inlineStr">
+      <c r="C84" s="23" t="inlineStr">
         <is>
           <t>The plan and the ninety days</t>
         </is>
       </c>
-      <c r="D84" s="14" t="inlineStr"/>
+      <c r="D84" s="16" t="inlineStr"/>
     </row>
     <row r="85">
-      <c r="A85" s="11" t="n">
+      <c r="A85" s="21" t="n">
         <v>81</v>
       </c>
-      <c r="B85" s="17" t="inlineStr">
+      <c r="B85" s="26" t="inlineStr">
         <is>
           <t>The Next Ninety</t>
         </is>
       </c>
-      <c r="C85" s="13" t="inlineStr">
+      <c r="C85" s="23" t="inlineStr">
         <is>
           <t>The plan and the ninety days</t>
         </is>
       </c>
-      <c r="D85" s="14" t="inlineStr"/>
+      <c r="D85" s="16" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" s="11" t="n">
+      <c r="A86" s="21" t="n">
         <v>82</v>
       </c>
-      <c r="B86" s="17" t="inlineStr">
+      <c r="B86" s="26" t="inlineStr">
         <is>
           <t>Day One</t>
         </is>
       </c>
-      <c r="C86" s="13" t="inlineStr">
+      <c r="C86" s="23" t="inlineStr">
         <is>
           <t>The plan and the ninety days</t>
         </is>
       </c>
-      <c r="D86" s="14" t="inlineStr"/>
-    </row>
-    <row r="87" ht="58" customHeight="1">
-      <c r="A87" s="11" t="n">
+      <c r="D86" s="16" t="inlineStr"/>
+    </row>
+    <row r="87" ht="30" customHeight="1">
+      <c r="A87" s="21" t="n">
         <v>83</v>
       </c>
-      <c r="B87" s="19" t="inlineStr">
+      <c r="B87" s="26" t="inlineStr">
         <is>
           <t>Gameplan</t>
         </is>
       </c>
-      <c r="C87" s="13" t="inlineStr">
+      <c r="C87" s="23" t="inlineStr">
         <is>
           <t>The plan and the ninety days</t>
         </is>
       </c>
-      <c r="D87" s="14" t="inlineStr">
-        <is>
-          <t>NOTE: Already the product's own word for the deliverable; using it as the company name would be redundant.</t>
+      <c r="D87" s="16" t="inlineStr">
+        <is>
+          <t>NOTE: Already the product's own word for the deliverable; redundant as a company name.</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="11" t="n">
+      <c r="A88" s="21" t="n">
         <v>84</v>
       </c>
-      <c r="B88" s="17" t="inlineStr">
+      <c r="B88" s="26" t="inlineStr">
         <is>
           <t>Blueprint</t>
         </is>
       </c>
-      <c r="C88" s="13" t="inlineStr">
+      <c r="C88" s="23" t="inlineStr">
         <is>
           <t>The plan and the ninety days</t>
         </is>
       </c>
-      <c r="D88" s="14" t="inlineStr"/>
+      <c r="D88" s="16" t="inlineStr"/>
     </row>
     <row r="89">
-      <c r="A89" s="11" t="n">
+      <c r="A89" s="21" t="n">
         <v>85</v>
       </c>
-      <c r="B89" s="17" t="inlineStr">
+      <c r="B89" s="26" t="inlineStr">
         <is>
           <t>Charter</t>
         </is>
       </c>
-      <c r="C89" s="13" t="inlineStr">
+      <c r="C89" s="23" t="inlineStr">
         <is>
           <t>The plan and the ninety days</t>
         </is>
       </c>
-      <c r="D89" s="14" t="inlineStr"/>
+      <c r="D89" s="16" t="inlineStr"/>
     </row>
     <row r="90">
-      <c r="A90" s="11" t="n">
+      <c r="A90" s="21" t="n">
         <v>86</v>
       </c>
-      <c r="B90" s="17" t="inlineStr">
+      <c r="B90" s="26" t="inlineStr">
         <is>
           <t>Groundwork</t>
         </is>
       </c>
-      <c r="C90" s="13" t="inlineStr">
+      <c r="C90" s="23" t="inlineStr">
         <is>
           <t>The plan and the ninety days</t>
         </is>
       </c>
-      <c r="D90" s="14" t="inlineStr"/>
+      <c r="D90" s="16" t="inlineStr"/>
     </row>
     <row r="91">
-      <c r="A91" s="11" t="n">
+      <c r="A91" s="21" t="n">
         <v>87</v>
       </c>
-      <c r="B91" s="17" t="inlineStr">
+      <c r="B91" s="26" t="inlineStr">
         <is>
           <t>Throughline</t>
         </is>
       </c>
-      <c r="C91" s="13" t="inlineStr">
+      <c r="C91" s="23" t="inlineStr">
         <is>
           <t>The plan and the ninety days</t>
         </is>
       </c>
-      <c r="D91" s="14" t="inlineStr"/>
+      <c r="D91" s="16" t="inlineStr"/>
     </row>
     <row r="92">
-      <c r="A92" s="11" t="n">
+      <c r="A92" s="21" t="n">
         <v>88</v>
       </c>
-      <c r="B92" s="17" t="inlineStr">
+      <c r="B92" s="26" t="inlineStr">
         <is>
           <t>Keystone</t>
         </is>
       </c>
-      <c r="C92" s="13" t="inlineStr">
+      <c r="C92" s="23" t="inlineStr">
         <is>
           <t>The plan and the ninety days</t>
         </is>
       </c>
-      <c r="D92" s="14" t="inlineStr"/>
+      <c r="D92" s="16" t="inlineStr"/>
     </row>
     <row r="93">
-      <c r="A93" s="11" t="n">
+      <c r="A93" s="21" t="n">
         <v>89</v>
       </c>
-      <c r="B93" s="17" t="inlineStr">
+      <c r="B93" s="26" t="inlineStr">
         <is>
           <t>Milestone</t>
         </is>
       </c>
-      <c r="C93" s="13" t="inlineStr">
+      <c r="C93" s="23" t="inlineStr">
         <is>
           <t>The plan and the ninety days</t>
         </is>
       </c>
-      <c r="D93" s="14" t="inlineStr"/>
+      <c r="D93" s="16" t="inlineStr"/>
     </row>
     <row r="94">
-      <c r="A94" s="11" t="n">
+      <c r="A94" s="21" t="n">
         <v>90</v>
       </c>
-      <c r="B94" s="17" t="inlineStr">
+      <c r="B94" s="26" t="inlineStr">
         <is>
           <t>Runway</t>
         </is>
       </c>
-      <c r="C94" s="13" t="inlineStr">
+      <c r="C94" s="23" t="inlineStr">
         <is>
           <t>The plan and the ninety days</t>
         </is>
       </c>
-      <c r="D94" s="14" t="inlineStr"/>
+      <c r="D94" s="16" t="inlineStr"/>
     </row>
     <row r="95">
-      <c r="A95" s="11" t="n">
+      <c r="A95" s="21" t="n">
         <v>91</v>
       </c>
-      <c r="B95" s="17" t="inlineStr">
+      <c r="B95" s="26" t="inlineStr">
         <is>
           <t>Plainly</t>
         </is>
       </c>
-      <c r="C95" s="13" t="inlineStr">
+      <c r="C95" s="23" t="inlineStr">
         <is>
           <t>Plain speech and proof</t>
         </is>
       </c>
-      <c r="D95" s="14" t="inlineStr"/>
+      <c r="D95" s="16" t="inlineStr"/>
     </row>
     <row r="96">
-      <c r="A96" s="11" t="n">
+      <c r="A96" s="21" t="n">
         <v>92</v>
       </c>
-      <c r="B96" s="17" t="inlineStr">
+      <c r="B96" s="26" t="inlineStr">
         <is>
           <t>Straight Answer</t>
         </is>
       </c>
-      <c r="C96" s="13" t="inlineStr">
+      <c r="C96" s="23" t="inlineStr">
         <is>
           <t>Plain speech and proof</t>
         </is>
       </c>
-      <c r="D96" s="14" t="inlineStr"/>
+      <c r="D96" s="16" t="inlineStr"/>
     </row>
     <row r="97">
-      <c r="A97" s="11" t="n">
+      <c r="A97" s="21" t="n">
         <v>93</v>
       </c>
-      <c r="B97" s="17" t="inlineStr">
+      <c r="B97" s="26" t="inlineStr">
         <is>
           <t>Cited</t>
         </is>
       </c>
-      <c r="C97" s="13" t="inlineStr">
+      <c r="C97" s="23" t="inlineStr">
         <is>
           <t>Plain speech and proof</t>
         </is>
       </c>
-      <c r="D97" s="14" t="inlineStr"/>
+      <c r="D97" s="16" t="inlineStr"/>
     </row>
     <row r="98">
-      <c r="A98" s="11" t="n">
+      <c r="A98" s="21" t="n">
         <v>94</v>
       </c>
-      <c r="B98" s="17" t="inlineStr">
+      <c r="B98" s="26" t="inlineStr">
         <is>
           <t>Sourced</t>
         </is>
       </c>
-      <c r="C98" s="13" t="inlineStr">
+      <c r="C98" s="23" t="inlineStr">
         <is>
           <t>Plain speech and proof</t>
         </is>
       </c>
-      <c r="D98" s="14" t="inlineStr"/>
+      <c r="D98" s="16" t="inlineStr"/>
     </row>
     <row r="99">
-      <c r="A99" s="11" t="n">
+      <c r="A99" s="21" t="n">
         <v>95</v>
       </c>
-      <c r="B99" s="17" t="inlineStr">
+      <c r="B99" s="26" t="inlineStr">
         <is>
           <t>Verified</t>
         </is>
       </c>
-      <c r="C99" s="13" t="inlineStr">
+      <c r="C99" s="23" t="inlineStr">
         <is>
           <t>Plain speech and proof</t>
         </is>
       </c>
-      <c r="D99" s="14" t="inlineStr"/>
+      <c r="D99" s="16" t="inlineStr"/>
     </row>
     <row r="100">
-      <c r="A100" s="11" t="n">
+      <c r="A100" s="21" t="n">
         <v>96</v>
       </c>
-      <c r="B100" s="17" t="inlineStr">
+      <c r="B100" s="26" t="inlineStr">
         <is>
           <t>Proof</t>
         </is>
       </c>
-      <c r="C100" s="13" t="inlineStr">
+      <c r="C100" s="23" t="inlineStr">
         <is>
           <t>Plain speech and proof</t>
         </is>
       </c>
-      <c r="D100" s="14" t="inlineStr"/>
+      <c r="D100" s="16" t="inlineStr"/>
     </row>
     <row r="101">
-      <c r="A101" s="11" t="n">
+      <c r="A101" s="21" t="n">
         <v>97</v>
       </c>
-      <c r="B101" s="17" t="inlineStr">
+      <c r="B101" s="26" t="inlineStr">
         <is>
           <t>Common Ground</t>
         </is>
       </c>
-      <c r="C101" s="13" t="inlineStr">
+      <c r="C101" s="23" t="inlineStr">
         <is>
           <t>Plain speech and proof</t>
         </is>
       </c>
-      <c r="D101" s="14" t="inlineStr"/>
-    </row>
-    <row r="102" ht="58" customHeight="1">
-      <c r="A102" s="11" t="n">
+      <c r="D101" s="16" t="inlineStr"/>
+    </row>
+    <row r="102" ht="30" customHeight="1">
+      <c r="A102" s="21" t="n">
         <v>98</v>
       </c>
-      <c r="B102" s="16" t="inlineStr">
+      <c r="B102" s="26" t="inlineStr">
         <is>
           <t>Anchor</t>
         </is>
       </c>
-      <c r="C102" s="13" t="inlineStr">
+      <c r="C102" s="23" t="inlineStr">
         <is>
           <t>Plain speech and proof</t>
         </is>
       </c>
-      <c r="D102" s="14" t="inlineStr">
+      <c r="D102" s="16" t="inlineStr">
         <is>
           <t>KNOWN CONFLICT: Anchor was a podcasting platform, acquired by Spotify.</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="11" t="n">
+      <c r="A103" s="21" t="n">
         <v>99</v>
       </c>
-      <c r="B103" s="17" t="inlineStr">
+      <c r="B103" s="26" t="inlineStr">
         <is>
           <t>Cornerstone</t>
         </is>
       </c>
-      <c r="C103" s="13" t="inlineStr">
+      <c r="C103" s="23" t="inlineStr">
         <is>
           <t>Plain speech and proof</t>
         </is>
       </c>
-      <c r="D103" s="14" t="inlineStr"/>
+      <c r="D103" s="16" t="inlineStr"/>
     </row>
     <row r="104">
-      <c r="A104" s="11" t="n">
+      <c r="A104" s="21" t="n">
         <v>100</v>
       </c>
-      <c r="B104" s="17" t="inlineStr">
+      <c r="B104" s="26" t="inlineStr">
         <is>
           <t>Foothold</t>
         </is>
       </c>
-      <c r="C104" s="13" t="inlineStr">
+      <c r="C104" s="23" t="inlineStr">
         <is>
           <t>Plain speech and proof</t>
         </is>
       </c>
-      <c r="D104" s="14" t="inlineStr"/>
+      <c r="D104" s="16" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2798,7 +3299,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2818,130 +3319,130 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
+    <row r="2" ht="44" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>These are naming patterns excluded on purpose, because they conflict with promises the product already makes.</t>
+          <t>Naming patterns excluded on purpose, because they conflict with promises the product already makes.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Pattern</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Why it is excluded</t>
         </is>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="28" t="inlineStr">
         <is>
           <t>VA, Federal, National, Official</t>
         </is>
       </c>
-      <c r="B5" s="21" t="inlineStr">
+      <c r="B5" s="29" t="inlineStr">
         <is>
           <t>Implies government affiliation. The product's central promise is that it is not the VA, and a name that muddies that is a liability, not a shortcut to credibility.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="20" t="inlineStr">
+      <c r="A6" s="28" t="inlineStr">
         <is>
           <t>Claims, Advocate, Counsel, Rep</t>
         </is>
       </c>
-      <c r="B6" s="21" t="inlineStr">
+      <c r="B6" s="29" t="inlineStr">
         <is>
           <t>Suggests accredited claims representation, which we are not and cannot imply. This is the one area with real regulatory teeth.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="20" t="inlineStr">
+      <c r="A7" s="28" t="inlineStr">
         <is>
           <t>Recruit, Enlist, Join Up</t>
         </is>
       </c>
-      <c r="B7" s="21" t="inlineStr">
+      <c r="B7" s="29" t="inlineStr">
         <is>
           <t>Reads as recruiting. The Reserve and Guard content already carries an explicit 'we are not recruiters, and no branch pays us' line. A name cannot undercut it.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="28" t="inlineStr">
         <is>
           <t>Guardian</t>
         </is>
       </c>
-      <c r="B8" s="21" t="inlineStr">
+      <c r="B8" s="29" t="inlineStr">
         <is>
           <t>Veterans Guardian is an existing paid-claims company, and Guardian is now the title for a Space Force member. Two collisions in one word.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="20" t="inlineStr">
+      <c r="A9" s="28" t="inlineStr">
         <is>
           <t>Patriot, Onward, Battle Buddy, Combined Arms</t>
         </is>
       </c>
-      <c r="B9" s="21" t="inlineStr">
-        <is>
-          <t>All occupied by organizations already in our competitive landscape. Patriot is also politically loaded in a way that costs us half a room.</t>
+      <c r="B9" s="29" t="inlineStr">
+        <is>
+          <t>All occupied by organisations already in our competitive landscape. Patriot is also politically loaded in a way that costs us half a room.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="20" t="inlineStr">
+      <c r="A10" s="28" t="inlineStr">
         <is>
           <t>Hero, Warrior, Brave</t>
         </is>
       </c>
-      <c r="B10" s="21" t="inlineStr">
+      <c r="B10" s="29" t="inlineStr">
         <is>
           <t>Many veterans find hero language cloying, and it signals a charity that wants to feel good about helping rather than a tool that respects them.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="20" t="inlineStr">
+      <c r="A11" s="28" t="inlineStr">
         <is>
           <t>Gold Star</t>
         </is>
       </c>
-      <c r="B11" s="21" t="inlineStr">
+      <c r="B11" s="29" t="inlineStr">
         <is>
           <t>Refers to the family of a service member who died. Never available for commercial use, in any framing.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1">
-      <c r="A12" s="20" t="inlineStr">
+      <c r="A12" s="28" t="inlineStr">
         <is>
           <t>Wounded, Disabled, Broken</t>
         </is>
       </c>
-      <c r="B12" s="21" t="inlineStr">
-        <is>
-          <t>Narrows a whole-life product to one chapter, and stigmatizes the veterans it claims to serve.</t>
+      <c r="B12" s="29" t="inlineStr">
+        <is>
+          <t>Narrows a whole-life product to one chapter, and stigmatises the veterans it claims to serve.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="58" customHeight="1">
-      <c r="A14" s="22" t="inlineStr">
-        <is>
-          <t>Caveat</t>
-        </is>
-      </c>
-      <c r="B14" s="23" t="inlineStr">
-        <is>
-          <t>This workbook is not a legal clearance opinion. USPTO full-text search blocked automated access, so registrations were pulled one at a time by serial number and coverage is partial by construction. Absence of a conflict means nothing was found, not that nothing exists. No WHOIS was run, so nothing here claims a domain is available. Before registering anything, a trademark attorney should run a real clearance search on the finalist.</t>
+      <c r="A14" s="30" t="inlineStr">
+        <is>
+          <t>Before registering anything</t>
+        </is>
+      </c>
+      <c r="B14" s="31" t="inlineStr">
+        <is>
+          <t>This workbook is not a legal clearance opinion. USPTO full-text search blocked automated access, so registrations were pulled one at a time by serial number and coverage is partial by construction. Absence of a conflict means nothing was found, not that nothing exists. No WHOIS was run, so nothing here claims a domain is available. A trademark attorney should run a real clearance search on the finalist before any money is spent.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add sample marks for the six strongest available names
The "Available now" tab gains a mark column for the top six. The ten earlier
marks on "Start here" are untouched: the workbook now carries sixteen, verified
present after the save.

Each mark comes from what its name means. Change of Station moves from an empty
post to a completed one. The Ground Ahead is a road running to the horizon.
Ninety Days Out is a ring split in thirds. Twelve Months Out is a twelve-cell
calendar with the first month lit. Order of March is a sequence of points with
the first one accented. The Next Ninety is a ninety-degree arc with the right
angle drawn in.

Two were redrawn after the first render. Twelve Months Out had twelve radial
ticks that read as a sun, which duplicated Reveille and said nothing about
months. The Ground Ahead had stacked contours that read as an arch rather than
terrain.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/share/VetPath-Naming-Candidates.xlsx
+++ b/share/VetPath-Naming-Candidates.xlsx
@@ -691,6 +691,161 @@
 </wsDr>
 </file>
 
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2238375" cy="647700"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2238375" cy="647700"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2238375" cy="647700"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2238375" cy="647700"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2238375" cy="647700"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2238375" cy="647700"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1342,14 +1497,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="84" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -1362,7 +1518,7 @@
     <row r="2" ht="62" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>A further 125 candidates were generated specifically to be registrable and checked against the registry before being shown here. Only these came back free. Every one below has BOTH the .com and the .org unregistered as of 29 July 2026, checked via Verisign and Public Interest Registry RDAP. IMPORTANT: an available domain is not a cleared name. None of these has had a trademark search, and the qualified variants at the bottom inherit whatever problem their parent name carries: adding 'Vets' to a domain does nothing about a live registration on the word itself.</t>
+          <t>A further 125 candidates were generated specifically to be registrable and checked against the registry before being shown here. Only these came back free. Every one below has BOTH the .com and the .org unregistered as of 29 July 2026, checked via Verisign and Public Interest Registry RDAP. The top six carry a sample mark. IMPORTANT: an available domain is not a cleared name. None of these has had a trademark search, and the qualified variants at the bottom inherit whatever problem their parent name carries: adding 'Vets' to a domain does nothing about a live registration on the word itself.</t>
         </is>
       </c>
     </row>
@@ -1374,540 +1530,565 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
+          <t>Sample mark</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>.com</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>.org</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Why, and what to watch</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="46" customHeight="1">
+    <row r="5" ht="62" customHeight="1">
       <c r="A5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="37" t="inlineStr">
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="37" t="inlineStr">
         <is>
           <t>Change of Station
 STRONG</t>
         </is>
       </c>
-      <c r="C5" s="38" t="inlineStr">
+      <c r="D5" s="38" t="inlineStr">
         <is>
           <t>changeofstation.com  FREE</t>
         </is>
       </c>
-      <c r="D5" s="38" t="inlineStr">
+      <c r="E5" s="38" t="inlineStr">
         <is>
           <t>changeofstation.org  FREE</t>
         </is>
       </c>
-      <c r="E5" s="39" t="inlineStr">
-        <is>
-          <t>Every service member knows PCS, and leaving the service is the biggest change of station there is. Plain, dignified, instantly legible to veterans without being jargon to anyone else. A search found no organisation using it as a brand.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="46" customHeight="1">
+      <c r="F5" s="39" t="inlineStr">
+        <is>
+          <t>Every service member knows PCS, and leaving the service is the biggest change of station there is. Plain, dignified, legible to veterans without being jargon to anyone else. A search found no organisation using it as a brand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="62" customHeight="1">
       <c r="A6" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="37" t="inlineStr">
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="37" t="inlineStr">
         <is>
           <t>The Ground Ahead
 STRONG</t>
         </is>
       </c>
-      <c r="C6" s="38" t="inlineStr">
+      <c r="D6" s="38" t="inlineStr">
         <is>
           <t>thegroundahead.com  FREE</t>
         </is>
       </c>
-      <c r="D6" s="38" t="inlineStr">
+      <c r="E6" s="38" t="inlineStr">
         <is>
           <t>thegroundahead.org  FREE</t>
         </is>
       </c>
-      <c r="E6" s="39" t="inlineStr">
+      <c r="F6" s="39" t="inlineStr">
         <is>
           <t>Plain, forward-looking, no military jargon at all, so it travels to spouses, grant officers and partners without translation.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="46" customHeight="1">
+    <row r="7" ht="62" customHeight="1">
       <c r="A7" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="37" t="inlineStr">
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="37" t="inlineStr">
         <is>
           <t>Ninety Days Out
 STRONG</t>
         </is>
       </c>
-      <c r="C7" s="38" t="inlineStr">
+      <c r="D7" s="38" t="inlineStr">
         <is>
           <t>ninetydaysout.com  FREE</t>
         </is>
       </c>
-      <c r="D7" s="38" t="inlineStr">
+      <c r="E7" s="38" t="inlineStr">
         <is>
           <t>ninetydaysout.org  FREE</t>
         </is>
       </c>
-      <c r="E7" s="39" t="inlineStr">
+      <c r="F7" s="39" t="inlineStr">
         <is>
           <t>Ties directly to the 30/60/90 plan the product actually produces. Says what it does.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="46" customHeight="1">
+    <row r="8" ht="62" customHeight="1">
       <c r="A8" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="37" t="inlineStr">
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="37" t="inlineStr">
         <is>
           <t>Twelve Months Out
 STRONG</t>
         </is>
       </c>
-      <c r="C8" s="38" t="inlineStr">
+      <c r="D8" s="38" t="inlineStr">
         <is>
           <t>twelvemonthsout.com  FREE</t>
         </is>
       </c>
-      <c r="D8" s="38" t="inlineStr">
+      <c r="E8" s="38" t="inlineStr">
         <is>
           <t>twelvemonthsout.org  FREE</t>
         </is>
       </c>
-      <c r="E8" s="39" t="inlineStr">
+      <c r="F8" s="39" t="inlineStr">
         <is>
           <t>Matches the primary user exactly: service members 0-24 months from separation.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="46" customHeight="1">
+    <row r="9" ht="62" customHeight="1">
       <c r="A9" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="37" t="inlineStr">
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="37" t="inlineStr">
         <is>
           <t>Order of March
 STRONG</t>
         </is>
       </c>
-      <c r="C9" s="38" t="inlineStr">
+      <c r="D9" s="38" t="inlineStr">
         <is>
           <t>orderofmarch.com  FREE</t>
         </is>
       </c>
-      <c r="D9" s="38" t="inlineStr">
+      <c r="E9" s="38" t="inlineStr">
         <is>
           <t>orderofmarch.org  FREE</t>
         </is>
       </c>
-      <c r="E9" s="39" t="inlineStr">
+      <c r="F9" s="39" t="inlineStr">
         <is>
           <t>The sequence in which a formation moves. Quietly military, and it means putting things in the right order, which is the product.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="46" customHeight="1">
+    <row r="10" ht="62" customHeight="1">
       <c r="A10" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="37" t="inlineStr">
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="37" t="inlineStr">
         <is>
           <t>The Next Ninety
 STRONG</t>
         </is>
       </c>
-      <c r="C10" s="38" t="inlineStr">
+      <c r="D10" s="38" t="inlineStr">
         <is>
           <t>thenextninety.com  FREE</t>
         </is>
       </c>
-      <c r="D10" s="38" t="inlineStr">
+      <c r="E10" s="38" t="inlineStr">
         <is>
           <t>thenextninety.org  FREE</t>
         </is>
       </c>
-      <c r="E10" s="39" t="inlineStr">
+      <c r="F10" s="39" t="inlineStr">
         <is>
           <t>Plain and tied to the deliverable.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="46" customHeight="1">
+    <row r="11" ht="44" customHeight="1">
       <c r="A11" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="40" t="inlineStr">
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="40" t="inlineStr">
         <is>
           <t>Operations Order
 WORKABLE</t>
         </is>
       </c>
-      <c r="C11" s="38" t="inlineStr">
+      <c r="D11" s="38" t="inlineStr">
         <is>
           <t>operationsorder.com  FREE</t>
         </is>
       </c>
-      <c r="D11" s="38" t="inlineStr">
+      <c r="E11" s="38" t="inlineStr">
         <is>
           <t>operationsorder.org  FREE</t>
         </is>
       </c>
-      <c r="E11" s="39" t="inlineStr">
+      <c r="F11" s="39" t="inlineStr">
         <is>
           <t>The five-paragraph order is the plan itself, so the meaning is exact. But it reads as jargon to civilians and to a grant officer.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="46" customHeight="1">
+    <row r="12" ht="44" customHeight="1">
       <c r="A12" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="40" t="inlineStr">
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="40" t="inlineStr">
         <is>
           <t>The Next Chapter Vets
 WORKABLE</t>
         </is>
       </c>
-      <c r="C12" s="38" t="inlineStr">
+      <c r="D12" s="38" t="inlineStr">
         <is>
           <t>thenextchaptervets.com  FREE</t>
         </is>
       </c>
-      <c r="D12" s="38" t="inlineStr">
+      <c r="E12" s="38" t="inlineStr">
         <is>
           <t>thenextchaptervets.org  FREE</t>
         </is>
       </c>
-      <c r="E12" s="39" t="inlineStr">
+      <c r="F12" s="39" t="inlineStr">
         <is>
           <t>Warm and clear, though 'next chapter' is heavily used in transition writing generally.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="46" customHeight="1">
+    <row r="13" ht="44" customHeight="1">
       <c r="A13" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="41" t="inlineStr">
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="41" t="inlineStr">
         <is>
           <t>Due North Vets
 QUALIFIED</t>
         </is>
       </c>
-      <c r="C13" s="38" t="inlineStr">
+      <c r="D13" s="38" t="inlineStr">
         <is>
           <t>duenorthvets.com  FREE</t>
         </is>
       </c>
-      <c r="D13" s="38" t="inlineStr">
+      <c r="E13" s="38" t="inlineStr">
         <is>
           <t>duenorthvets.org  FREE</t>
         </is>
       </c>
-      <c r="E13" s="39" t="inlineStr">
+      <c r="F13" s="39" t="inlineStr">
         <is>
           <t>Keeps the cleanest name and gets a real domain.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="46" customHeight="1">
+    <row r="14" ht="44" customHeight="1">
       <c r="A14" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="41" t="inlineStr">
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="41" t="inlineStr">
         <is>
           <t>Due North Veterans
 QUALIFIED</t>
         </is>
       </c>
-      <c r="C14" s="38" t="inlineStr">
+      <c r="D14" s="38" t="inlineStr">
         <is>
           <t>duenorthveterans.com  FREE</t>
         </is>
       </c>
-      <c r="D14" s="38" t="inlineStr">
+      <c r="E14" s="38" t="inlineStr">
         <is>
           <t>duenorthveterans.org  FREE</t>
         </is>
       </c>
-      <c r="E14" s="39" t="inlineStr">
+      <c r="F14" s="39" t="inlineStr">
         <is>
           <t>As above, spelled out.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="46" customHeight="1">
+    <row r="15" ht="44" customHeight="1">
       <c r="A15" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="41" t="inlineStr">
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="41" t="inlineStr">
         <is>
           <t>Get Due North
 QUALIFIED</t>
         </is>
       </c>
-      <c r="C15" s="38" t="inlineStr">
+      <c r="D15" s="38" t="inlineStr">
         <is>
           <t>getduenorth.com  FREE</t>
         </is>
       </c>
-      <c r="D15" s="38" t="inlineStr">
+      <c r="E15" s="38" t="inlineStr">
         <is>
           <t>getduenorth.org  FREE</t>
         </is>
       </c>
-      <c r="E15" s="39" t="inlineStr">
+      <c r="F15" s="39" t="inlineStr">
         <is>
           <t>Verb form. Reads as a call to action.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="46" customHeight="1">
+    <row r="16" ht="44" customHeight="1">
       <c r="A16" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="41" t="inlineStr">
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="41" t="inlineStr">
         <is>
           <t>Due North Planning
 QUALIFIED</t>
         </is>
       </c>
-      <c r="C16" s="38" t="inlineStr">
+      <c r="D16" s="38" t="inlineStr">
         <is>
           <t>duenorthplanning.com  FREE</t>
         </is>
       </c>
-      <c r="D16" s="38" t="inlineStr">
+      <c r="E16" s="38" t="inlineStr">
         <is>
           <t>duenorthplanning.org  FREE</t>
         </is>
       </c>
-      <c r="E16" s="39" t="inlineStr">
+      <c r="F16" s="39" t="inlineStr">
         <is>
           <t>Says the category outright.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="46" customHeight="1">
+    <row r="17" ht="44" customHeight="1">
       <c r="A17" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="41" t="inlineStr">
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="41" t="inlineStr">
         <is>
           <t>Due North Gameplan
 QUALIFIED</t>
         </is>
       </c>
-      <c r="C17" s="38" t="inlineStr">
+      <c r="D17" s="38" t="inlineStr">
         <is>
           <t>duenorthgameplan.com  FREE</t>
         </is>
       </c>
-      <c r="D17" s="38" t="inlineStr">
+      <c r="E17" s="38" t="inlineStr">
         <is>
           <t>duenorthgameplan.org  FREE</t>
         </is>
       </c>
-      <c r="E17" s="39" t="inlineStr">
+      <c r="F17" s="39" t="inlineStr">
         <is>
           <t>Uses the product's own word for the deliverable.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="46" customHeight="1">
+    <row r="18" ht="44" customHeight="1">
       <c r="A18" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="41" t="inlineStr">
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="41" t="inlineStr">
         <is>
           <t>Lodestar Vets
 QUALIFIED</t>
         </is>
       </c>
-      <c r="C18" s="38" t="inlineStr">
+      <c r="D18" s="38" t="inlineStr">
         <is>
           <t>lodestarvets.com  FREE</t>
         </is>
       </c>
-      <c r="D18" s="38" t="inlineStr">
+      <c r="E18" s="38" t="inlineStr">
         <is>
           <t>lodestarvets.org  FREE</t>
         </is>
       </c>
-      <c r="E18" s="39" t="inlineStr">
+      <c r="F18" s="39" t="inlineStr">
         <is>
           <t>Keeps the name with the cleanest veteran space.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="46" customHeight="1">
+    <row r="19" ht="44" customHeight="1">
       <c r="A19" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="41" t="inlineStr">
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="41" t="inlineStr">
         <is>
           <t>Lodestar Veterans
 QUALIFIED</t>
         </is>
       </c>
-      <c r="C19" s="38" t="inlineStr">
+      <c r="D19" s="38" t="inlineStr">
         <is>
           <t>lodestarveterans.com  FREE</t>
         </is>
       </c>
-      <c r="D19" s="38" t="inlineStr">
+      <c r="E19" s="38" t="inlineStr">
         <is>
           <t>lodestarveterans.org  FREE</t>
         </is>
       </c>
-      <c r="E19" s="39" t="inlineStr">
+      <c r="F19" s="39" t="inlineStr">
         <is>
           <t>As above, spelled out.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="46" customHeight="1">
+    <row r="20" ht="44" customHeight="1">
       <c r="A20" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="41" t="inlineStr">
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="41" t="inlineStr">
         <is>
           <t>Lodestar Planning
 QUALIFIED</t>
         </is>
       </c>
-      <c r="C20" s="38" t="inlineStr">
+      <c r="D20" s="38" t="inlineStr">
         <is>
           <t>lodestarplanning.com  FREE</t>
         </is>
       </c>
-      <c r="D20" s="38" t="inlineStr">
+      <c r="E20" s="38" t="inlineStr">
         <is>
           <t>lodestarplanning.org  FREE</t>
         </is>
       </c>
-      <c r="E20" s="39" t="inlineStr">
-        <is>
-          <t>Note: Lodestar has a live Class 36 mark for investment advisory, so a planning-flavoured name is the riskier qualifier here.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="46" customHeight="1">
+      <c r="F20" s="39" t="inlineStr">
+        <is>
+          <t>Note: Lodestar has a live Class 36 mark for investment advisory, so a planning-flavoured qualifier is the riskier choice here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="44" customHeight="1">
       <c r="A21" s="5" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="41" t="inlineStr">
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="41" t="inlineStr">
         <is>
           <t>Lodestar Gameplan
 QUALIFIED</t>
         </is>
       </c>
-      <c r="C21" s="38" t="inlineStr">
+      <c r="D21" s="38" t="inlineStr">
         <is>
           <t>lodestargameplan.com  FREE</t>
         </is>
       </c>
-      <c r="D21" s="38" t="inlineStr">
+      <c r="E21" s="38" t="inlineStr">
         <is>
           <t>lodestargameplan.org  FREE</t>
         </is>
       </c>
-      <c r="E21" s="39" t="inlineStr">
+      <c r="F21" s="39" t="inlineStr">
         <is>
           <t>Safer qualifier than Planning, given that Class 36 mark.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="46" customHeight="1">
+    <row r="22" ht="44" customHeight="1">
       <c r="A22" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="41" t="inlineStr">
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="41" t="inlineStr">
         <is>
           <t>After Action Vets
 QUALIFIED</t>
         </is>
       </c>
-      <c r="C22" s="38" t="inlineStr">
+      <c r="D22" s="38" t="inlineStr">
         <is>
           <t>afteractionvets.com  FREE</t>
         </is>
       </c>
-      <c r="D22" s="38" t="inlineStr">
+      <c r="E22" s="38" t="inlineStr">
         <is>
           <t>afteractionvets.org  FREE</t>
         </is>
       </c>
-      <c r="E22" s="39" t="inlineStr">
+      <c r="F22" s="39" t="inlineStr">
         <is>
           <t>Inherits the weak-distinctiveness problem of the parent name.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="46" customHeight="1">
+    <row r="23" ht="44" customHeight="1">
       <c r="A23" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="41" t="inlineStr">
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="41" t="inlineStr">
         <is>
           <t>Earned Vets
 QUALIFIED</t>
         </is>
       </c>
-      <c r="C23" s="38" t="inlineStr">
+      <c r="D23" s="38" t="inlineStr">
         <is>
           <t>earnedvets.com  FREE</t>
         </is>
       </c>
-      <c r="D23" s="38" t="inlineStr">
+      <c r="E23" s="38" t="inlineStr">
         <is>
           <t>earnedvets.org  FREE</t>
         </is>
       </c>
-      <c r="E23" s="39" t="inlineStr">
+      <c r="F23" s="39" t="inlineStr">
         <is>
           <t>Inherits the parent's search problem: 'earned benefits' is everywhere in VA writing.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="46" customHeight="1">
+    <row r="24" ht="44" customHeight="1">
       <c r="A24" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="41" t="inlineStr">
+      <c r="B24" s="6" t="n"/>
+      <c r="C24" s="41" t="inlineStr">
         <is>
           <t>Reveille Vets
 QUALIFIED</t>
         </is>
       </c>
-      <c r="C24" s="38" t="inlineStr">
+      <c r="D24" s="38" t="inlineStr">
         <is>
           <t>reveillevets.com  FREE</t>
         </is>
       </c>
-      <c r="D24" s="38" t="inlineStr">
+      <c r="E24" s="38" t="inlineStr">
         <is>
           <t>reveillevets.org  FREE</t>
         </is>
       </c>
-      <c r="E24" s="39" t="inlineStr">
+      <c r="F24" s="39" t="inlineStr">
         <is>
           <t>Inherits the parent's real problem: a live Class 41 registration for veteran education. Listed for completeness, not recommended.</t>
         </is>
@@ -1915,9 +2096,10 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A2:F2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Warm recolor for brand assets: OG card, PWA icons, print PDFs, logo marks
The site went warm (green/amber) earlier; this carries the palette into
everything that renders outside the app itself:

- scripts/og-card.html + public/og-card.jpg regenerated at 1200x630
- PWA icons (192/512/apple-touch) rebuilt: amber route tile on deep green
- manifest theme_color/background_color and layout.tsx themeColor updated
- all five print/*.html palettes swapped and PDFs regenerated
  (page counts unchanged: 3/4/12/2/2)
- demo static-fallback brand mark warmed (last navy literal in the mirror)
- naming workbook sample marks re-rendered in the warm palette

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/share/VetPath-Naming-Candidates.xlsx
+++ b/share/VetPath-Naming-Candidates.xlsx
@@ -714,6 +714,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -739,6 +742,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -764,6 +770,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -789,6 +798,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -814,6 +826,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -839,6 +854,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>

</xml_diff>